<commit_message>
Add 11 new Nate Claude Code tutorials to challenge days + update tracker
New videos added as placeholders (youtube: null) across Days 1-6:
- Day 1: How I'd Teach a 10 Year Old, Zero to Your First CC Workflow
- Day 2: Firecrawl - Scrape Anything, Nano Banana 2 + Claude Code
- Day 3: Claude Code Skills, Claude Code Skills Just Got Even Better
- Day 4: Website Building 5 Hacks, CC + Trigger.dev
- Day 6: CC Executive Assistant, Watch My AI Agents Work, CC Remote Control

Tracker rebuilt: 91 items across 8 days.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Progress Tracker Template.xlsx
+++ b/Progress Tracker Template.xlsx
@@ -588,10 +588,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D134"/>
+  <dimension ref="A1:D145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="60" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
@@ -614,12 +614,12 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>#</t>
+          <t>ID</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Section</t>
+          <t>Type</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -811,7 +811,7 @@
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>CH-102</t>
+          <t>CC-NEW-01</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -821,7 +821,7 @@
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>🎬 Installing &amp; Configuring Claude Code</t>
+          <t>🎬 How I'd Teach a 10 Year Old</t>
         </is>
       </c>
       <c r="D18" s="8" t="b">
@@ -831,17 +831,17 @@
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>CH-103</t>
+          <t>CC-NEW-02</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>Lesson</t>
+          <t>Video</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>📖 The Claude Code Build Loop</t>
+          <t>🎬 Zero to Your First CC Workflow</t>
         </is>
       </c>
       <c r="D19" s="8" t="b">
@@ -849,214 +849,214 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Build</t>
-        </is>
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>CH-102</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>Video</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>🎬 Installing &amp; Configuring Claude Code</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
+          <t>CH-103</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>📖 The Claude Code Build Loop</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Build</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
           <t>CH-104</t>
         </is>
       </c>
-      <c r="B21" s="6" t="inlineStr">
+      <c r="B23" s="6" t="inlineStr">
         <is>
           <t>Build</t>
         </is>
       </c>
-      <c r="C21" s="7" t="inlineStr">
+      <c r="C23" s="7" t="inlineStr">
         <is>
           <t>🔨 Project: Build a CLI Task Manager</t>
         </is>
       </c>
-      <c r="D21" s="8" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="6" t="inlineStr">
-        <is>
-          <t>CH-105</t>
-        </is>
-      </c>
-      <c r="B22" s="6" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="C22" s="7" t="inlineStr">
-        <is>
-          <t>🔨 Bonus Build: Personal Expense Tracker</t>
-        </is>
-      </c>
-      <c r="D22" s="8" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Reference</t>
-        </is>
+      <c r="D23" s="8" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
+          <t>CH-105</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>🔨 Bonus Build: Personal Expense Tracker</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Reference</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
           <t>CH-106</t>
         </is>
       </c>
-      <c r="B24" s="6" t="inlineStr">
+      <c r="B26" s="6" t="inlineStr">
         <is>
           <t>Resource</t>
         </is>
       </c>
-      <c r="C24" s="7" t="inlineStr">
+      <c r="C26" s="7" t="inlineStr">
         <is>
           <t>📋 Claude Code Cheat Sheet</t>
         </is>
       </c>
-      <c r="D24" s="8" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="6" t="inlineStr">
-        <is>
-          <t>CH-107</t>
-        </is>
-      </c>
-      <c r="B25" s="6" t="inlineStr">
-        <is>
-          <t>Lesson</t>
-        </is>
-      </c>
-      <c r="C25" s="7" t="inlineStr">
-        <is>
-          <t>📖 Troubleshooting: Common Day 1 Issues</t>
-        </is>
-      </c>
-      <c r="D25" s="8" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Checkpoint</t>
-        </is>
+      <c r="D26" s="8" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
+          <t>CH-107</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>📖 Troubleshooting: Common Day 1 Issues</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Checkpoint</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
           <t>CH-108</t>
         </is>
       </c>
-      <c r="B27" s="6" t="inlineStr">
+      <c r="B29" s="6" t="inlineStr">
         <is>
           <t>Quiz</t>
         </is>
       </c>
-      <c r="C27" s="7" t="inlineStr">
+      <c r="C29" s="7" t="inlineStr">
         <is>
           <t>❓ Day 1 Knowledge Check</t>
         </is>
       </c>
-      <c r="D27" s="8" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="6" t="inlineStr">
+      <c r="D29" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
         <is>
           <t>CH-109</t>
         </is>
       </c>
-      <c r="B28" s="6" t="inlineStr">
+      <c r="B30" s="6" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="C28" s="7" t="inlineStr">
+      <c r="C30" s="7" t="inlineStr">
         <is>
           <t>📢 Share Your Day 1 Build</t>
         </is>
       </c>
-      <c r="D28" s="8" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" ht="28" customHeight="1">
-      <c r="A30" s="10" t="inlineStr">
+      <c r="D30" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" ht="28" customHeight="1">
+      <c r="A32" s="10" t="inlineStr">
         <is>
           <t>Day 2: AI-Powered Applications</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="5" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">  Learn</t>
         </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="6" t="inlineStr">
-        <is>
-          <t>CH-201</t>
-        </is>
-      </c>
-      <c r="B32" s="6" t="inlineStr">
-        <is>
-          <t>Lesson</t>
-        </is>
-      </c>
-      <c r="C32" s="7" t="inlineStr">
-        <is>
-          <t>📖 Working with AI APIs Through Claude Code</t>
-        </is>
-      </c>
-      <c r="D32" s="8" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="6" t="inlineStr">
-        <is>
-          <t>CH-202</t>
-        </is>
-      </c>
-      <c r="B33" s="6" t="inlineStr">
-        <is>
-          <t>Lesson</t>
-        </is>
-      </c>
-      <c r="C33" s="7" t="inlineStr">
-        <is>
-          <t>📖 Giving Claude Code Context That Matters</t>
-        </is>
-      </c>
-      <c r="D33" s="8" t="b">
-        <v>0</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>CH-203</t>
+          <t>CC-NEW-03</t>
         </is>
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>Lesson</t>
+          <t>Video</t>
         </is>
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>📖 Iterative Building: Start Simple, Then Layer</t>
+          <t>🎬 Firecrawl - Scrape Anything</t>
         </is>
       </c>
       <c r="D34" s="8" t="b">
@@ -1064,26 +1064,39 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Build</t>
-        </is>
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>CC-NEW-04</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="inlineStr">
+        <is>
+          <t>Video</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>🎬 Nano Banana 2 + Claude Code</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>CH-204</t>
+          <t>CH-201</t>
         </is>
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>Build</t>
+          <t>Lesson</t>
         </is>
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>🔨 Project: AI Content Generator</t>
+          <t>📖 Working with AI APIs Through Claude Code</t>
         </is>
       </c>
       <c r="D36" s="8" t="b">
@@ -1093,17 +1106,17 @@
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>CH-205</t>
+          <t>CH-202</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>Build</t>
+          <t>Lesson</t>
         </is>
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>🔨 Alternate Build: Smart URL Summarizer</t>
+          <t>📖 Giving Claude Code Context That Matters</t>
         </is>
       </c>
       <c r="D37" s="8" t="b">
@@ -1113,17 +1126,17 @@
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>CH-206</t>
+          <t>CH-203</t>
         </is>
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>Build</t>
+          <t>Lesson</t>
         </is>
       </c>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>🔨 Alternate Build: Data Analysis Assistant</t>
+          <t>📖 Iterative Building: Start Simple, Then Layer</t>
         </is>
       </c>
       <c r="D38" s="8" t="b">
@@ -1133,24 +1146,24 @@
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Go Deeper</t>
+          <t xml:space="preserve">  Build</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>CH-207</t>
+          <t>CH-204</t>
         </is>
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>Lesson</t>
+          <t>Build</t>
         </is>
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>📖 Environment Variables &amp; API Key Security</t>
+          <t>🔨 Project: AI Content Generator</t>
         </is>
       </c>
       <c r="D40" s="8" t="b">
@@ -1160,17 +1173,17 @@
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>CH-208</t>
+          <t>CH-205</t>
         </is>
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>Lesson</t>
+          <t>Build</t>
         </is>
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>📖 Adding Error Handling &amp; Loading States</t>
+          <t>🔨 Alternate Build: Smart URL Summarizer</t>
         </is>
       </c>
       <c r="D41" s="8" t="b">
@@ -1178,167 +1191,167 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Checkpoint</t>
-        </is>
+      <c r="A42" s="6" t="inlineStr">
+        <is>
+          <t>CH-206</t>
+        </is>
+      </c>
+      <c r="B42" s="6" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="C42" s="7" t="inlineStr">
+        <is>
+          <t>🔨 Alternate Build: Data Analysis Assistant</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="6" t="inlineStr">
-        <is>
-          <t>CH-209</t>
-        </is>
-      </c>
-      <c r="B43" s="6" t="inlineStr">
-        <is>
-          <t>Quiz</t>
-        </is>
-      </c>
-      <c r="C43" s="7" t="inlineStr">
-        <is>
-          <t>❓ Day 2 Knowledge Check</t>
-        </is>
-      </c>
-      <c r="D43" s="8" t="b">
-        <v>0</v>
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Go Deeper</t>
+        </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>CH-210</t>
+          <t>CH-207</t>
         </is>
       </c>
       <c r="B44" s="6" t="inlineStr">
         <is>
-          <t>Action</t>
+          <t>Lesson</t>
         </is>
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>📢 Share Your Day 2 Build</t>
+          <t>📖 Environment Variables &amp; API Key Security</t>
         </is>
       </c>
       <c r="D44" s="8" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="46" ht="28" customHeight="1">
-      <c r="A46" s="11" t="inlineStr">
-        <is>
-          <t>Day 3: Master Claude Code</t>
+    <row r="45">
+      <c r="A45" s="6" t="inlineStr">
+        <is>
+          <t>CH-208</t>
+        </is>
+      </c>
+      <c r="B45" s="6" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="C45" s="7" t="inlineStr">
+        <is>
+          <t>📖 Adding Error Handling &amp; Loading States</t>
+        </is>
+      </c>
+      <c r="D45" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Checkpoint</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Learn</t>
-        </is>
+      <c r="A47" s="6" t="inlineStr">
+        <is>
+          <t>CH-209</t>
+        </is>
+      </c>
+      <c r="B47" s="6" t="inlineStr">
+        <is>
+          <t>Quiz</t>
+        </is>
+      </c>
+      <c r="C47" s="7" t="inlineStr">
+        <is>
+          <t>❓ Day 2 Knowledge Check</t>
+        </is>
+      </c>
+      <c r="D47" s="8" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t>CC-003</t>
+          <t>CH-210</t>
         </is>
       </c>
       <c r="B48" s="6" t="inlineStr">
         <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="C48" s="7" t="inlineStr">
+        <is>
+          <t>📢 Share Your Day 2 Build</t>
+        </is>
+      </c>
+      <c r="D48" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" ht="28" customHeight="1">
+      <c r="A50" s="11" t="inlineStr">
+        <is>
+          <t>Day 3: Master Claude Code</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Learn</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="6" t="inlineStr">
+        <is>
+          <t>CC-NEW-05</t>
+        </is>
+      </c>
+      <c r="B52" s="6" t="inlineStr">
+        <is>
           <t>Video</t>
         </is>
       </c>
-      <c r="C48" s="7" t="inlineStr">
-        <is>
-          <t>🎬 Master 95% of Claude Code (Video)</t>
-        </is>
-      </c>
-      <c r="D48" s="8" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="6" t="inlineStr">
-        <is>
-          <t>CH-301</t>
-        </is>
-      </c>
-      <c r="B49" s="6" t="inlineStr">
-        <is>
-          <t>Lesson</t>
-        </is>
-      </c>
-      <c r="C49" s="7" t="inlineStr">
-        <is>
-          <t>📖 CLAUDE.md: Your Project's Brain</t>
-        </is>
-      </c>
-      <c r="D49" s="8" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="6" t="inlineStr">
-        <is>
-          <t>CH-302</t>
-        </is>
-      </c>
-      <c r="B50" s="6" t="inlineStr">
-        <is>
-          <t>Lesson</t>
-        </is>
-      </c>
-      <c r="C50" s="7" t="inlineStr">
-        <is>
-          <t>📖 Prompt Patterns That Work</t>
-        </is>
-      </c>
-      <c r="D50" s="8" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="6" t="inlineStr">
-        <is>
-          <t>CH-303</t>
-        </is>
-      </c>
-      <c r="B51" s="6" t="inlineStr">
-        <is>
-          <t>Lesson</t>
-        </is>
-      </c>
-      <c r="C51" s="7" t="inlineStr">
-        <is>
-          <t>📖 Multi-File Projects &amp; Code Organization</t>
-        </is>
-      </c>
-      <c r="D51" s="8" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Build</t>
-        </is>
+      <c r="C52" s="7" t="inlineStr">
+        <is>
+          <t>🎬 Claude Code Skills</t>
+        </is>
+      </c>
+      <c r="D52" s="8" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>CH-304</t>
+          <t>CC-NEW-06</t>
         </is>
       </c>
       <c r="B53" s="6" t="inlineStr">
         <is>
-          <t>Build</t>
+          <t>Video</t>
         </is>
       </c>
       <c r="C53" s="7" t="inlineStr">
         <is>
-          <t>🔨 Project: Three Mini-Builds, Three Techniques</t>
+          <t>🎬 Claude Code Skills Just Got Even Better</t>
         </is>
       </c>
       <c r="D53" s="8" t="b">
@@ -1348,17 +1361,17 @@
     <row r="54">
       <c r="A54" s="6" t="inlineStr">
         <is>
-          <t>CH-305</t>
+          <t>CC-003</t>
         </is>
       </c>
       <c r="B54" s="6" t="inlineStr">
         <is>
-          <t>Build</t>
+          <t>Video</t>
         </is>
       </c>
       <c r="C54" s="7" t="inlineStr">
         <is>
-          <t>🔨 Create Your First CLAUDE.md</t>
+          <t>🎬 Master 95% of Claude Code</t>
         </is>
       </c>
       <c r="D54" s="8" t="b">
@@ -1366,16 +1379,29 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Go Deeper</t>
-        </is>
+      <c r="A55" s="6" t="inlineStr">
+        <is>
+          <t>CH-301</t>
+        </is>
+      </c>
+      <c r="B55" s="6" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="C55" s="7" t="inlineStr">
+        <is>
+          <t>📖 CLAUDE.md: Your Project's Brain</t>
+        </is>
+      </c>
+      <c r="D55" s="8" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="6" t="inlineStr">
         <is>
-          <t>CH-306</t>
+          <t>CH-302</t>
         </is>
       </c>
       <c r="B56" s="6" t="inlineStr">
@@ -1385,7 +1411,7 @@
       </c>
       <c r="C56" s="7" t="inlineStr">
         <is>
-          <t>📖 Git Integration with Claude Code</t>
+          <t>📖 Prompt Patterns That Work</t>
         </is>
       </c>
       <c r="D56" s="8" t="b">
@@ -1395,7 +1421,7 @@
     <row r="57">
       <c r="A57" s="6" t="inlineStr">
         <is>
-          <t>CH-307</t>
+          <t>CH-303</t>
         </is>
       </c>
       <c r="B57" s="6" t="inlineStr">
@@ -1405,7 +1431,7 @@
       </c>
       <c r="C57" s="7" t="inlineStr">
         <is>
-          <t>📖 Debugging with Claude Code</t>
+          <t>📖 Multi-File Projects &amp; Code Organization</t>
         </is>
       </c>
       <c r="D57" s="8" t="b">
@@ -1415,24 +1441,24 @@
     <row r="58">
       <c r="A58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Checkpoint</t>
+          <t xml:space="preserve">  Build</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="6" t="inlineStr">
         <is>
-          <t>CH-308</t>
+          <t>CH-304</t>
         </is>
       </c>
       <c r="B59" s="6" t="inlineStr">
         <is>
-          <t>Quiz</t>
+          <t>Build</t>
         </is>
       </c>
       <c r="C59" s="7" t="inlineStr">
         <is>
-          <t>❓ Day 3 Knowledge Check</t>
+          <t>🔨 Project: Three Mini-Builds, Three Techniques</t>
         </is>
       </c>
       <c r="D59" s="8" t="b">
@@ -1442,71 +1468,91 @@
     <row r="60">
       <c r="A60" s="6" t="inlineStr">
         <is>
-          <t>CH-309</t>
+          <t>CH-305</t>
         </is>
       </c>
       <c r="B60" s="6" t="inlineStr">
         <is>
-          <t>Action</t>
+          <t>Build</t>
         </is>
       </c>
       <c r="C60" s="7" t="inlineStr">
         <is>
-          <t>📢 Share Your Day 3 Builds</t>
+          <t>🔨 Create Your First CLAUDE.md</t>
         </is>
       </c>
       <c r="D60" s="8" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="62" ht="28" customHeight="1">
-      <c r="A62" s="12" t="inlineStr">
-        <is>
-          <t>Day 4: Full-Stack Web Applications</t>
-        </is>
+    <row r="61">
+      <c r="A61" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Go Deeper</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="6" t="inlineStr">
+        <is>
+          <t>CH-306</t>
+        </is>
+      </c>
+      <c r="B62" s="6" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="C62" s="7" t="inlineStr">
+        <is>
+          <t>📖 Git Integration with Claude Code</t>
+        </is>
+      </c>
+      <c r="D62" s="8" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Learn</t>
-        </is>
+      <c r="A63" s="6" t="inlineStr">
+        <is>
+          <t>CH-307</t>
+        </is>
+      </c>
+      <c r="B63" s="6" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="C63" s="7" t="inlineStr">
+        <is>
+          <t>📖 Debugging with Claude Code</t>
+        </is>
+      </c>
+      <c r="D63" s="8" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="6" t="inlineStr">
-        <is>
-          <t>CH-401</t>
-        </is>
-      </c>
-      <c r="B64" s="6" t="inlineStr">
-        <is>
-          <t>Lesson</t>
-        </is>
-      </c>
-      <c r="C64" s="7" t="inlineStr">
-        <is>
-          <t>📖 Claude Code for Full-Stack Development</t>
-        </is>
-      </c>
-      <c r="D64" s="8" t="b">
-        <v>0</v>
+      <c r="A64" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Checkpoint</t>
+        </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>CH-402</t>
+          <t>CH-308</t>
         </is>
       </c>
       <c r="B65" s="6" t="inlineStr">
         <is>
-          <t>Lesson</t>
+          <t>Quiz</t>
         </is>
       </c>
       <c r="C65" s="7" t="inlineStr">
         <is>
-          <t>📖 The Product Spec Approach</t>
+          <t>❓ Day 3 Knowledge Check</t>
         </is>
       </c>
       <c r="D65" s="8" t="b">
@@ -1516,84 +1562,51 @@
     <row r="66">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>CH-403</t>
+          <t>CH-309</t>
         </is>
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>Lesson</t>
+          <t>Action</t>
         </is>
       </c>
       <c r="C66" s="7" t="inlineStr">
         <is>
-          <t>📖 Databases with Claude Code</t>
+          <t>📢 Share Your Day 3 Builds</t>
         </is>
       </c>
       <c r="D66" s="8" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Build</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="6" t="inlineStr">
-        <is>
-          <t>CH-404</t>
-        </is>
-      </c>
-      <c r="B68" s="6" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="C68" s="7" t="inlineStr">
-        <is>
-          <t>🔨 Project: Build a Full-Stack Dashboard App</t>
-        </is>
-      </c>
-      <c r="D68" s="8" t="b">
-        <v>0</v>
+    <row r="68" ht="28" customHeight="1">
+      <c r="A68" s="12" t="inlineStr">
+        <is>
+          <t>Day 4: Full-Stack Web Applications</t>
+        </is>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="6" t="inlineStr">
-        <is>
-          <t>CH-405</t>
-        </is>
-      </c>
-      <c r="B69" s="6" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="C69" s="7" t="inlineStr">
-        <is>
-          <t>🔨 Alternate Build: SaaS Landing Page with Auth</t>
-        </is>
-      </c>
-      <c r="D69" s="8" t="b">
-        <v>0</v>
+      <c r="A69" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Learn</t>
+        </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>CH-406</t>
+          <t>CC-NEW-07</t>
         </is>
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>Build</t>
+          <t>Video</t>
         </is>
       </c>
       <c r="C70" s="7" t="inlineStr">
         <is>
-          <t>🔨 Alternate Build: API with Documentation</t>
+          <t>🎬 Website Building 5 Hacks</t>
         </is>
       </c>
       <c r="D70" s="8" t="b">
@@ -1601,16 +1614,29 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Go Deeper</t>
-        </is>
+      <c r="A71" s="6" t="inlineStr">
+        <is>
+          <t>CC-NEW-08</t>
+        </is>
+      </c>
+      <c r="B71" s="6" t="inlineStr">
+        <is>
+          <t>Video</t>
+        </is>
+      </c>
+      <c r="C71" s="7" t="inlineStr">
+        <is>
+          <t>🎬 CC + Trigger.dev</t>
+        </is>
+      </c>
+      <c r="D71" s="8" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>CH-407</t>
+          <t>CH-401</t>
         </is>
       </c>
       <c r="B72" s="6" t="inlineStr">
@@ -1620,7 +1646,7 @@
       </c>
       <c r="C72" s="7" t="inlineStr">
         <is>
-          <t>📖 Deploying Your App to Vercel</t>
+          <t>📖 Claude Code for Full-Stack Development</t>
         </is>
       </c>
       <c r="D72" s="8" t="b">
@@ -1630,7 +1656,7 @@
     <row r="73">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>CH-408</t>
+          <t>CH-402</t>
         </is>
       </c>
       <c r="B73" s="6" t="inlineStr">
@@ -1640,7 +1666,7 @@
       </c>
       <c r="C73" s="7" t="inlineStr">
         <is>
-          <t>📖 Adding Real-Time Features</t>
+          <t>📖 The Product Spec Approach</t>
         </is>
       </c>
       <c r="D73" s="8" t="b">
@@ -1648,70 +1674,103 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Checkpoint</t>
-        </is>
+      <c r="A74" s="6" t="inlineStr">
+        <is>
+          <t>CH-403</t>
+        </is>
+      </c>
+      <c r="B74" s="6" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="C74" s="7" t="inlineStr">
+        <is>
+          <t>📖 Databases with Claude Code</t>
+        </is>
+      </c>
+      <c r="D74" s="8" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="6" t="inlineStr">
-        <is>
-          <t>CH-409</t>
-        </is>
-      </c>
-      <c r="B75" s="6" t="inlineStr">
-        <is>
-          <t>Quiz</t>
-        </is>
-      </c>
-      <c r="C75" s="7" t="inlineStr">
-        <is>
-          <t>❓ Day 4 Knowledge Check</t>
-        </is>
-      </c>
-      <c r="D75" s="8" t="b">
-        <v>0</v>
+      <c r="A75" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Build</t>
+        </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="6" t="inlineStr">
         <is>
-          <t>CH-410</t>
+          <t>CH-404</t>
         </is>
       </c>
       <c r="B76" s="6" t="inlineStr">
         <is>
-          <t>Action</t>
+          <t>Build</t>
         </is>
       </c>
       <c r="C76" s="7" t="inlineStr">
         <is>
-          <t>📢 Share Your Day 4 Build</t>
+          <t>🔨 Project: Build a Full-Stack Dashboard App</t>
         </is>
       </c>
       <c r="D76" s="8" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="78" ht="28" customHeight="1">
-      <c r="A78" s="13" t="inlineStr">
-        <is>
-          <t>Day 5: RAG &amp; AI Agent Systems</t>
-        </is>
+    <row r="77">
+      <c r="A77" s="6" t="inlineStr">
+        <is>
+          <t>CH-405</t>
+        </is>
+      </c>
+      <c r="B77" s="6" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="C77" s="7" t="inlineStr">
+        <is>
+          <t>🔨 Alternate Build: SaaS Landing Page with Auth</t>
+        </is>
+      </c>
+      <c r="D77" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="6" t="inlineStr">
+        <is>
+          <t>CH-406</t>
+        </is>
+      </c>
+      <c r="B78" s="6" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="C78" s="7" t="inlineStr">
+        <is>
+          <t>🔨 Alternate Build: API with Documentation</t>
+        </is>
+      </c>
+      <c r="D78" s="8" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Learn</t>
+          <t xml:space="preserve">  Go Deeper</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="6" t="inlineStr">
         <is>
-          <t>CH-501</t>
+          <t>CH-407</t>
         </is>
       </c>
       <c r="B80" s="6" t="inlineStr">
@@ -1721,7 +1780,7 @@
       </c>
       <c r="C80" s="7" t="inlineStr">
         <is>
-          <t>📖 What is RAG and Why Every Business Wants It</t>
+          <t>📖 Deploying Your App to Vercel</t>
         </is>
       </c>
       <c r="D80" s="8" t="b">
@@ -1731,7 +1790,7 @@
     <row r="81">
       <c r="A81" s="6" t="inlineStr">
         <is>
-          <t>CH-502</t>
+          <t>CH-408</t>
         </is>
       </c>
       <c r="B81" s="6" t="inlineStr">
@@ -1741,7 +1800,7 @@
       </c>
       <c r="C81" s="7" t="inlineStr">
         <is>
-          <t>📖 The RAG Pipeline: How It Works</t>
+          <t>📖 Adding Real-Time Features</t>
         </is>
       </c>
       <c r="D81" s="8" t="b">
@@ -1749,103 +1808,70 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="6" t="inlineStr">
-        <is>
-          <t>CH-503</t>
-        </is>
-      </c>
-      <c r="B82" s="6" t="inlineStr">
-        <is>
-          <t>Lesson</t>
-        </is>
-      </c>
-      <c r="C82" s="7" t="inlineStr">
-        <is>
-          <t>📖 Choosing a Vector Database</t>
-        </is>
-      </c>
-      <c r="D82" s="8" t="b">
-        <v>0</v>
+      <c r="A82" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Checkpoint</t>
+        </is>
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Build</t>
-        </is>
+      <c r="A83" s="6" t="inlineStr">
+        <is>
+          <t>CH-409</t>
+        </is>
+      </c>
+      <c r="B83" s="6" t="inlineStr">
+        <is>
+          <t>Quiz</t>
+        </is>
+      </c>
+      <c r="C83" s="7" t="inlineStr">
+        <is>
+          <t>❓ Day 4 Knowledge Check</t>
+        </is>
+      </c>
+      <c r="D83" s="8" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="6" t="inlineStr">
         <is>
-          <t>CH-504</t>
+          <t>CH-410</t>
         </is>
       </c>
       <c r="B84" s="6" t="inlineStr">
         <is>
-          <t>Build</t>
+          <t>Action</t>
         </is>
       </c>
       <c r="C84" s="7" t="inlineStr">
         <is>
-          <t>🔨 Project: Chat With Your Documents</t>
+          <t>📢 Share Your Day 4 Build</t>
         </is>
       </c>
       <c r="D84" s="8" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="85">
-      <c r="A85" s="6" t="inlineStr">
-        <is>
-          <t>CH-505</t>
-        </is>
-      </c>
-      <c r="B85" s="6" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="C85" s="7" t="inlineStr">
-        <is>
-          <t>🔨 Alternate Build: Research Assistant Agent</t>
-        </is>
-      </c>
-      <c r="D85" s="8" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" s="6" t="inlineStr">
-        <is>
-          <t>CH-506</t>
-        </is>
-      </c>
-      <c r="B86" s="6" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="C86" s="7" t="inlineStr">
-        <is>
-          <t>🔨 Alternate Build: Q&amp;A Bot for Knowledge Base</t>
-        </is>
-      </c>
-      <c r="D86" s="8" t="b">
-        <v>0</v>
+    <row r="86" ht="28" customHeight="1">
+      <c r="A86" s="13" t="inlineStr">
+        <is>
+          <t>Day 5: RAG &amp; AI Agent Systems</t>
+        </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Go Deeper</t>
+          <t xml:space="preserve">  Learn</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="6" t="inlineStr">
         <is>
-          <t>CH-507</t>
+          <t>CH-501</t>
         </is>
       </c>
       <c r="B88" s="6" t="inlineStr">
@@ -1855,7 +1881,7 @@
       </c>
       <c r="C88" s="7" t="inlineStr">
         <is>
-          <t>📖 Chunking Strategies That Matter</t>
+          <t>📖 What is RAG and Why Every Business Wants It</t>
         </is>
       </c>
       <c r="D88" s="8" t="b">
@@ -1865,7 +1891,7 @@
     <row r="89">
       <c r="A89" s="6" t="inlineStr">
         <is>
-          <t>CH-508</t>
+          <t>CH-502</t>
         </is>
       </c>
       <c r="B89" s="6" t="inlineStr">
@@ -1875,7 +1901,7 @@
       </c>
       <c r="C89" s="7" t="inlineStr">
         <is>
-          <t>📖 Adding Memory to Your AI</t>
+          <t>📖 The RAG Pipeline: How It Works</t>
         </is>
       </c>
       <c r="D89" s="8" t="b">
@@ -1885,7 +1911,7 @@
     <row r="90">
       <c r="A90" s="6" t="inlineStr">
         <is>
-          <t>CH-509</t>
+          <t>CH-503</t>
         </is>
       </c>
       <c r="B90" s="6" t="inlineStr">
@@ -1895,7 +1921,7 @@
       </c>
       <c r="C90" s="7" t="inlineStr">
         <is>
-          <t>📖 Evaluating RAG Quality</t>
+          <t>📖 Choosing a Vector Database</t>
         </is>
       </c>
       <c r="D90" s="8" t="b">
@@ -1905,24 +1931,24 @@
     <row r="91">
       <c r="A91" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Checkpoint</t>
+          <t xml:space="preserve">  Build</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="6" t="inlineStr">
         <is>
-          <t>CH-510</t>
+          <t>CH-504</t>
         </is>
       </c>
       <c r="B92" s="6" t="inlineStr">
         <is>
-          <t>Quiz</t>
+          <t>Build</t>
         </is>
       </c>
       <c r="C92" s="7" t="inlineStr">
         <is>
-          <t>❓ Day 5 Knowledge Check</t>
+          <t>🔨 Project: Chat With Your Documents</t>
         </is>
       </c>
       <c r="D92" s="8" t="b">
@@ -1932,41 +1958,74 @@
     <row r="93">
       <c r="A93" s="6" t="inlineStr">
         <is>
-          <t>CH-511</t>
+          <t>CH-505</t>
         </is>
       </c>
       <c r="B93" s="6" t="inlineStr">
         <is>
-          <t>Action</t>
+          <t>Build</t>
         </is>
       </c>
       <c r="C93" s="7" t="inlineStr">
         <is>
-          <t>📢 Share Your Day 5 Build</t>
+          <t>🔨 Alternate Build: Research Assistant Agent</t>
         </is>
       </c>
       <c r="D93" s="8" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="95" ht="28" customHeight="1">
-      <c r="A95" s="14" t="inlineStr">
-        <is>
-          <t>Day 6: Complex Multi-Component Projects</t>
+    <row r="94">
+      <c r="A94" s="6" t="inlineStr">
+        <is>
+          <t>CH-506</t>
+        </is>
+      </c>
+      <c r="B94" s="6" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="C94" s="7" t="inlineStr">
+        <is>
+          <t>🔨 Alternate Build: Q&amp;A Bot for Knowledge Base</t>
+        </is>
+      </c>
+      <c r="D94" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Go Deeper</t>
         </is>
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Learn</t>
-        </is>
+      <c r="A96" s="6" t="inlineStr">
+        <is>
+          <t>CH-507</t>
+        </is>
+      </c>
+      <c r="B96" s="6" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="C96" s="7" t="inlineStr">
+        <is>
+          <t>📖 Chunking Strategies That Matter</t>
+        </is>
+      </c>
+      <c r="D96" s="8" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="6" t="inlineStr">
         <is>
-          <t>CH-601</t>
+          <t>CH-508</t>
         </is>
       </c>
       <c r="B97" s="6" t="inlineStr">
@@ -1976,7 +2035,7 @@
       </c>
       <c r="C97" s="7" t="inlineStr">
         <is>
-          <t>📖 Thinking in Systems, Not Scripts</t>
+          <t>📖 Adding Memory to Your AI</t>
         </is>
       </c>
       <c r="D97" s="8" t="b">
@@ -1986,7 +2045,7 @@
     <row r="98">
       <c r="A98" s="6" t="inlineStr">
         <is>
-          <t>CH-602</t>
+          <t>CH-509</t>
         </is>
       </c>
       <c r="B98" s="6" t="inlineStr">
@@ -1996,7 +2055,7 @@
       </c>
       <c r="C98" s="7" t="inlineStr">
         <is>
-          <t>📖 API Design Patterns</t>
+          <t>📖 Evaluating RAG Quality</t>
         </is>
       </c>
       <c r="D98" s="8" t="b">
@@ -2004,113 +2063,80 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="6" t="inlineStr">
-        <is>
-          <t>CH-603</t>
-        </is>
-      </c>
-      <c r="B99" s="6" t="inlineStr">
-        <is>
-          <t>Lesson</t>
-        </is>
-      </c>
-      <c r="C99" s="7" t="inlineStr">
-        <is>
-          <t>📖 Working with External Services</t>
-        </is>
-      </c>
-      <c r="D99" s="8" t="b">
-        <v>0</v>
+      <c r="A99" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Checkpoint</t>
+        </is>
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Build</t>
-        </is>
+      <c r="A100" s="6" t="inlineStr">
+        <is>
+          <t>CH-510</t>
+        </is>
+      </c>
+      <c r="B100" s="6" t="inlineStr">
+        <is>
+          <t>Quiz</t>
+        </is>
+      </c>
+      <c r="C100" s="7" t="inlineStr">
+        <is>
+          <t>❓ Day 5 Knowledge Check</t>
+        </is>
+      </c>
+      <c r="D100" s="8" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="6" t="inlineStr">
         <is>
-          <t>CH-604</t>
+          <t>CH-511</t>
         </is>
       </c>
       <c r="B101" s="6" t="inlineStr">
         <is>
-          <t>Build</t>
+          <t>Action</t>
         </is>
       </c>
       <c r="C101" s="7" t="inlineStr">
         <is>
-          <t>🔨 Project: Multi-Service Application</t>
+          <t>📢 Share Your Day 5 Build</t>
         </is>
       </c>
       <c r="D101" s="8" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="102">
-      <c r="A102" s="6" t="inlineStr">
-        <is>
-          <t>CH-605</t>
-        </is>
-      </c>
-      <c r="B102" s="6" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="C102" s="7" t="inlineStr">
-        <is>
-          <t>🔨 Alternate Build: Slack Bot</t>
-        </is>
-      </c>
-      <c r="D102" s="8" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" s="6" t="inlineStr">
-        <is>
-          <t>CH-606</t>
-        </is>
-      </c>
-      <c r="B103" s="6" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="C103" s="7" t="inlineStr">
-        <is>
-          <t>🔨 Alternate Build: Chrome Extension</t>
-        </is>
-      </c>
-      <c r="D103" s="8" t="b">
-        <v>0</v>
+    <row r="103" ht="28" customHeight="1">
+      <c r="A103" s="14" t="inlineStr">
+        <is>
+          <t>Day 6: Complex Multi-Component Projects</t>
+        </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Go Deeper</t>
+          <t xml:space="preserve">  Learn</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="6" t="inlineStr">
         <is>
-          <t>CH-607</t>
+          <t>CC-NEW-09</t>
         </is>
       </c>
       <c r="B105" s="6" t="inlineStr">
         <is>
-          <t>Lesson</t>
+          <t>Video</t>
         </is>
       </c>
       <c r="C105" s="7" t="inlineStr">
         <is>
-          <t>📖 Testing Your Code with Claude Code</t>
+          <t>🎬 Claude Code Executive Assistant</t>
         </is>
       </c>
       <c r="D105" s="8" t="b">
@@ -2120,17 +2146,17 @@
     <row r="106">
       <c r="A106" s="6" t="inlineStr">
         <is>
-          <t>CH-608</t>
+          <t>CC-NEW-10</t>
         </is>
       </c>
       <c r="B106" s="6" t="inlineStr">
         <is>
-          <t>Lesson</t>
+          <t>Video</t>
         </is>
       </c>
       <c r="C106" s="7" t="inlineStr">
         <is>
-          <t>📖 Error Handling &amp; Logging</t>
+          <t>🎬 Watch My AI Agents Work in Real Time</t>
         </is>
       </c>
       <c r="D106" s="8" t="b">
@@ -2140,17 +2166,17 @@
     <row r="107">
       <c r="A107" s="6" t="inlineStr">
         <is>
-          <t>CH-609</t>
+          <t>CC-NEW-11</t>
         </is>
       </c>
       <c r="B107" s="6" t="inlineStr">
         <is>
-          <t>Lesson</t>
+          <t>Video</t>
         </is>
       </c>
       <c r="C107" s="7" t="inlineStr">
         <is>
-          <t>📖 Rate Limiting &amp; Security Basics</t>
+          <t>🎬 Claude Code Remote Control</t>
         </is>
       </c>
       <c r="D107" s="8" t="b">
@@ -2158,26 +2184,39 @@
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Checkpoint</t>
-        </is>
+      <c r="A108" s="6" t="inlineStr">
+        <is>
+          <t>CH-601</t>
+        </is>
+      </c>
+      <c r="B108" s="6" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="C108" s="7" t="inlineStr">
+        <is>
+          <t>📖 Thinking in Systems, Not Scripts</t>
+        </is>
+      </c>
+      <c r="D108" s="8" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="6" t="inlineStr">
         <is>
-          <t>CH-610</t>
+          <t>CH-602</t>
         </is>
       </c>
       <c r="B109" s="6" t="inlineStr">
         <is>
-          <t>Quiz</t>
+          <t>Lesson</t>
         </is>
       </c>
       <c r="C109" s="7" t="inlineStr">
         <is>
-          <t>❓ Day 6 Knowledge Check</t>
+          <t>📖 API Design Patterns</t>
         </is>
       </c>
       <c r="D109" s="8" t="b">
@@ -2187,51 +2226,84 @@
     <row r="110">
       <c r="A110" s="6" t="inlineStr">
         <is>
-          <t>CH-611</t>
+          <t>CH-603</t>
         </is>
       </c>
       <c r="B110" s="6" t="inlineStr">
         <is>
-          <t>Action</t>
+          <t>Lesson</t>
         </is>
       </c>
       <c r="C110" s="7" t="inlineStr">
         <is>
-          <t>📢 Share Your Day 6 Build</t>
+          <t>📖 Working with External Services</t>
         </is>
       </c>
       <c r="D110" s="8" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="112" ht="28" customHeight="1">
-      <c r="A112" s="15" t="inlineStr">
-        <is>
-          <t>Day 7: Production-Grade Capstone</t>
-        </is>
+    <row r="111">
+      <c r="A111" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Build</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="6" t="inlineStr">
+        <is>
+          <t>CH-604</t>
+        </is>
+      </c>
+      <c r="B112" s="6" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="C112" s="7" t="inlineStr">
+        <is>
+          <t>🔨 Project: Multi-Service Application</t>
+        </is>
+      </c>
+      <c r="D112" s="8" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Learn</t>
-        </is>
+      <c r="A113" s="6" t="inlineStr">
+        <is>
+          <t>CH-605</t>
+        </is>
+      </c>
+      <c r="B113" s="6" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="C113" s="7" t="inlineStr">
+        <is>
+          <t>🔨 Alternate Build: Slack Bot</t>
+        </is>
+      </c>
+      <c r="D113" s="8" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="6" t="inlineStr">
         <is>
-          <t>CH-701</t>
+          <t>CH-606</t>
         </is>
       </c>
       <c r="B114" s="6" t="inlineStr">
         <is>
-          <t>Lesson</t>
+          <t>Build</t>
         </is>
       </c>
       <c r="C114" s="7" t="inlineStr">
         <is>
-          <t>📖 What Makes Something Production-Grade</t>
+          <t>🔨 Alternate Build: Chrome Extension</t>
         </is>
       </c>
       <c r="D114" s="8" t="b">
@@ -2239,29 +2311,16 @@
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="6" t="inlineStr">
-        <is>
-          <t>CH-702</t>
-        </is>
-      </c>
-      <c r="B115" s="6" t="inlineStr">
-        <is>
-          <t>Lesson</t>
-        </is>
-      </c>
-      <c r="C115" s="7" t="inlineStr">
-        <is>
-          <t>📖 Documentation That Sells Your Work</t>
-        </is>
-      </c>
-      <c r="D115" s="8" t="b">
-        <v>0</v>
+      <c r="A115" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Go Deeper</t>
+        </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="6" t="inlineStr">
         <is>
-          <t>CH-703</t>
+          <t>CH-607</t>
         </is>
       </c>
       <c r="B116" s="6" t="inlineStr">
@@ -2271,7 +2330,7 @@
       </c>
       <c r="C116" s="7" t="inlineStr">
         <is>
-          <t>📖 CI/CD and Automated Deployment</t>
+          <t>📖 Testing Your Code with Claude Code</t>
         </is>
       </c>
       <c r="D116" s="8" t="b">
@@ -2279,26 +2338,39 @@
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Build</t>
-        </is>
+      <c r="A117" s="6" t="inlineStr">
+        <is>
+          <t>CH-608</t>
+        </is>
+      </c>
+      <c r="B117" s="6" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="C117" s="7" t="inlineStr">
+        <is>
+          <t>📖 Error Handling &amp; Logging</t>
+        </is>
+      </c>
+      <c r="D117" s="8" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="6" t="inlineStr">
         <is>
-          <t>CH-704</t>
+          <t>CH-609</t>
         </is>
       </c>
       <c r="B118" s="6" t="inlineStr">
         <is>
-          <t>Build</t>
+          <t>Lesson</t>
         </is>
       </c>
       <c r="C118" s="7" t="inlineStr">
         <is>
-          <t>🔨 Capstone: Make Your Best Project Production-Ready</t>
+          <t>📖 Rate Limiting &amp; Security Basics</t>
         </is>
       </c>
       <c r="D118" s="8" t="b">
@@ -2306,39 +2378,26 @@
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="6" t="inlineStr">
-        <is>
-          <t>CH-705</t>
-        </is>
-      </c>
-      <c r="B119" s="6" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="C119" s="7" t="inlineStr">
-        <is>
-          <t>🔨 Add a Feature You've Been Wanting</t>
-        </is>
-      </c>
-      <c r="D119" s="8" t="b">
-        <v>0</v>
+      <c r="A119" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Checkpoint</t>
+        </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="6" t="inlineStr">
         <is>
-          <t>CH-706</t>
+          <t>CH-610</t>
         </is>
       </c>
       <c r="B120" s="6" t="inlineStr">
         <is>
-          <t>Build</t>
+          <t>Quiz</t>
         </is>
       </c>
       <c r="C120" s="7" t="inlineStr">
         <is>
-          <t>🔨 Code Review: Ask Claude to Review Your Code</t>
+          <t>❓ Day 6 Knowledge Check</t>
         </is>
       </c>
       <c r="D120" s="8" t="b">
@@ -2346,93 +2405,73 @@
       </c>
     </row>
     <row r="121">
-      <c r="A121" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Go Deeper</t>
-        </is>
-      </c>
-    </row>
-    <row r="122">
-      <c r="A122" s="6" t="inlineStr">
-        <is>
-          <t>CH-707</t>
-        </is>
-      </c>
-      <c r="B122" s="6" t="inlineStr">
-        <is>
-          <t>Lesson</t>
-        </is>
-      </c>
-      <c r="C122" s="7" t="inlineStr">
-        <is>
-          <t>📖 Performance Optimization</t>
-        </is>
-      </c>
-      <c r="D122" s="8" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" s="6" t="inlineStr">
-        <is>
-          <t>CH-708</t>
-        </is>
-      </c>
-      <c r="B123" s="6" t="inlineStr">
-        <is>
-          <t>Lesson</t>
-        </is>
-      </c>
-      <c r="C123" s="7" t="inlineStr">
-        <is>
-          <t>📖 Monitoring &amp; Health Checks</t>
-        </is>
-      </c>
-      <c r="D123" s="8" t="b">
-        <v>0</v>
+      <c r="A121" s="6" t="inlineStr">
+        <is>
+          <t>CH-611</t>
+        </is>
+      </c>
+      <c r="B121" s="6" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="C121" s="7" t="inlineStr">
+        <is>
+          <t>📢 Share Your Day 6 Build</t>
+        </is>
+      </c>
+      <c r="D121" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="123" ht="28" customHeight="1">
+      <c r="A123" s="15" t="inlineStr">
+        <is>
+          <t>Day 7: Production-Grade Capstone</t>
+        </is>
       </c>
     </row>
     <row r="124">
-      <c r="A124" s="6" t="inlineStr">
-        <is>
-          <t>CH-709</t>
-        </is>
-      </c>
-      <c r="B124" s="6" t="inlineStr">
-        <is>
-          <t>Lesson</t>
-        </is>
-      </c>
-      <c r="C124" s="7" t="inlineStr">
-        <is>
-          <t>📖 Preparing for a Portfolio</t>
-        </is>
-      </c>
-      <c r="D124" s="8" t="b">
-        <v>0</v>
+      <c r="A124" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Learn</t>
+        </is>
       </c>
     </row>
     <row r="125">
-      <c r="A125" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Challenge Complete</t>
-        </is>
+      <c r="A125" s="6" t="inlineStr">
+        <is>
+          <t>CH-701</t>
+        </is>
+      </c>
+      <c r="B125" s="6" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="C125" s="7" t="inlineStr">
+        <is>
+          <t>📖 What Makes Something Production-Grade</t>
+        </is>
+      </c>
+      <c r="D125" s="8" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="6" t="inlineStr">
         <is>
-          <t>CH-710</t>
+          <t>CH-702</t>
         </is>
       </c>
       <c r="B126" s="6" t="inlineStr">
         <is>
-          <t>Quiz</t>
+          <t>Lesson</t>
         </is>
       </c>
       <c r="C126" s="7" t="inlineStr">
         <is>
-          <t>❓ Day 7 Knowledge Check (Final)</t>
+          <t>📖 Documentation That Sells Your Work</t>
         </is>
       </c>
       <c r="D126" s="8" t="b">
@@ -2442,17 +2481,17 @@
     <row r="127">
       <c r="A127" s="6" t="inlineStr">
         <is>
-          <t>CH-711</t>
+          <t>CH-703</t>
         </is>
       </c>
       <c r="B127" s="6" t="inlineStr">
         <is>
-          <t>Action</t>
+          <t>Lesson</t>
         </is>
       </c>
       <c r="C127" s="7" t="inlineStr">
         <is>
-          <t>📢 Submit Your Capstone</t>
+          <t>📖 CI/CD and Automated Deployment</t>
         </is>
       </c>
       <c r="D127" s="8" t="b">
@@ -2460,110 +2499,291 @@
       </c>
     </row>
     <row r="128">
-      <c r="A128" s="6" t="inlineStr">
-        <is>
-          <t>CH-712</t>
-        </is>
-      </c>
-      <c r="B128" s="6" t="inlineStr">
-        <is>
-          <t>Reward</t>
-        </is>
-      </c>
-      <c r="C128" s="7" t="inlineStr">
-        <is>
-          <t>🏆 Claim Your Challenge Rewards</t>
-        </is>
-      </c>
-      <c r="D128" s="8" t="b">
-        <v>0</v>
+      <c r="A128" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Build</t>
+        </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="6" t="inlineStr">
         <is>
+          <t>CH-704</t>
+        </is>
+      </c>
+      <c r="B129" s="6" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="C129" s="7" t="inlineStr">
+        <is>
+          <t>🔨 Capstone: Make Your Best Project Production-Ready</t>
+        </is>
+      </c>
+      <c r="D129" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="6" t="inlineStr">
+        <is>
+          <t>CH-705</t>
+        </is>
+      </c>
+      <c r="B130" s="6" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="C130" s="7" t="inlineStr">
+        <is>
+          <t>🔨 Add a Feature You've Been Wanting</t>
+        </is>
+      </c>
+      <c r="D130" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="6" t="inlineStr">
+        <is>
+          <t>CH-706</t>
+        </is>
+      </c>
+      <c r="B131" s="6" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="C131" s="7" t="inlineStr">
+        <is>
+          <t>🔨 Code Review: Ask Claude to Review Your Code</t>
+        </is>
+      </c>
+      <c r="D131" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Go Deeper</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="6" t="inlineStr">
+        <is>
+          <t>CH-707</t>
+        </is>
+      </c>
+      <c r="B133" s="6" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="C133" s="7" t="inlineStr">
+        <is>
+          <t>📖 Performance Optimization</t>
+        </is>
+      </c>
+      <c r="D133" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="6" t="inlineStr">
+        <is>
+          <t>CH-708</t>
+        </is>
+      </c>
+      <c r="B134" s="6" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="C134" s="7" t="inlineStr">
+        <is>
+          <t>📖 Monitoring &amp; Health Checks</t>
+        </is>
+      </c>
+      <c r="D134" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="6" t="inlineStr">
+        <is>
+          <t>CH-709</t>
+        </is>
+      </c>
+      <c r="B135" s="6" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="C135" s="7" t="inlineStr">
+        <is>
+          <t>📖 Preparing for a Portfolio</t>
+        </is>
+      </c>
+      <c r="D135" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Challenge Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="6" t="inlineStr">
+        <is>
+          <t>CH-710</t>
+        </is>
+      </c>
+      <c r="B137" s="6" t="inlineStr">
+        <is>
+          <t>Quiz</t>
+        </is>
+      </c>
+      <c r="C137" s="7" t="inlineStr">
+        <is>
+          <t>❓ Day 7 Knowledge Check (Final)</t>
+        </is>
+      </c>
+      <c r="D137" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="6" t="inlineStr">
+        <is>
+          <t>CH-711</t>
+        </is>
+      </c>
+      <c r="B138" s="6" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="C138" s="7" t="inlineStr">
+        <is>
+          <t>📢 Submit Your Capstone</t>
+        </is>
+      </c>
+      <c r="D138" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="6" t="inlineStr">
+        <is>
+          <t>CH-712</t>
+        </is>
+      </c>
+      <c r="B139" s="6" t="inlineStr">
+        <is>
+          <t>Reward</t>
+        </is>
+      </c>
+      <c r="C139" s="7" t="inlineStr">
+        <is>
+          <t>🏆 Claim Your Challenge Rewards</t>
+        </is>
+      </c>
+      <c r="D139" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="6" t="inlineStr">
+        <is>
           <t>CH-713</t>
         </is>
       </c>
-      <c r="B129" s="6" t="inlineStr">
-        <is>
-          <t>Lesson</t>
-        </is>
-      </c>
-      <c r="C129" s="7" t="inlineStr">
+      <c r="B140" s="6" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="C140" s="7" t="inlineStr">
         <is>
           <t>📖 Your Path Forward</t>
         </is>
       </c>
-      <c r="D129" s="8" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="132">
-      <c r="A132" s="16" t="inlineStr">
+      <c r="D140" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="16" t="inlineStr">
         <is>
           <t>REWARD ELIGIBILITY</t>
         </is>
       </c>
     </row>
-    <row r="133" ht="35" customHeight="1">
-      <c r="A133" s="17">
-        <f>IF(AND(D21=TRUE,D36=TRUE,D53=TRUE,D68=TRUE,D84=TRUE,D101=TRUE,D118=TRUE),"🏆 Ready to Claim!","Keep building — complete the main build for each day")</f>
+    <row r="144" ht="35" customHeight="1">
+      <c r="A144" s="17">
+        <f>IF(AND(D23=TRUE,D40=TRUE,D59=TRUE,D76=TRUE,D92=TRUE,D112=TRUE,D129=TRUE),"🏆 Ready to Claim!","Keep building — complete the main build for each day")</f>
         <v/>
       </c>
     </row>
-    <row r="134">
-      <c r="A134" s="18" t="inlineStr">
-        <is>
-          <t>Main builds tracked: Day 1 (row 21), Day 2 (row 36), Day 3 (row 53), Day 4 (row 68), Day 5 (row 84), Day 6 (row 101), Day 7 (row 118)</t>
+    <row r="145">
+      <c r="A145" s="18" t="inlineStr">
+        <is>
+          <t>Main builds tracked: Day 1 (row 23), Day 2 (row 40), Day 3 (row 59), Day 4 (row 76), Day 5 (row 92), Day 6 (row 112), Day 7 (row 129)</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="43">
     <mergeCell ref="A5:D5"/>
-    <mergeCell ref="A23:D23"/>
+    <mergeCell ref="A144:D144"/>
+    <mergeCell ref="A22:D22"/>
     <mergeCell ref="A91:D91"/>
-    <mergeCell ref="A35:D35"/>
-    <mergeCell ref="A62:D62"/>
-    <mergeCell ref="A20:D20"/>
-    <mergeCell ref="A96:D96"/>
-    <mergeCell ref="A100:D100"/>
-    <mergeCell ref="A52:D52"/>
-    <mergeCell ref="A134:D134"/>
-    <mergeCell ref="A112:D112"/>
-    <mergeCell ref="A125:D125"/>
-    <mergeCell ref="A63:D63"/>
-    <mergeCell ref="A121:D121"/>
-    <mergeCell ref="A117:D117"/>
-    <mergeCell ref="A67:D67"/>
-    <mergeCell ref="A31:D31"/>
+    <mergeCell ref="A43:D43"/>
+    <mergeCell ref="A28:D28"/>
+    <mergeCell ref="A115:D115"/>
+    <mergeCell ref="A68:D68"/>
+    <mergeCell ref="A111:D111"/>
     <mergeCell ref="A58:D58"/>
-    <mergeCell ref="A83:D83"/>
-    <mergeCell ref="A30:D30"/>
+    <mergeCell ref="A143:D143"/>
     <mergeCell ref="A39:D39"/>
     <mergeCell ref="A15:D15"/>
+    <mergeCell ref="A64:D64"/>
+    <mergeCell ref="A82:D82"/>
+    <mergeCell ref="A51:D51"/>
     <mergeCell ref="A11:D11"/>
+    <mergeCell ref="A123:D123"/>
     <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A103:D103"/>
     <mergeCell ref="A132:D132"/>
     <mergeCell ref="A79:D79"/>
+    <mergeCell ref="A61:D61"/>
     <mergeCell ref="A6:D6"/>
-    <mergeCell ref="A78:D78"/>
+    <mergeCell ref="A119:D119"/>
+    <mergeCell ref="A69:D69"/>
+    <mergeCell ref="A124:D124"/>
     <mergeCell ref="A87:D87"/>
+    <mergeCell ref="A25:D25"/>
+    <mergeCell ref="A128:D128"/>
     <mergeCell ref="A16:D16"/>
+    <mergeCell ref="A99:D99"/>
     <mergeCell ref="A46:D46"/>
-    <mergeCell ref="A133:D133"/>
-    <mergeCell ref="A108:D108"/>
-    <mergeCell ref="A74:D74"/>
-    <mergeCell ref="A26:D26"/>
-    <mergeCell ref="A55:D55"/>
+    <mergeCell ref="A75:D75"/>
+    <mergeCell ref="A136:D136"/>
+    <mergeCell ref="A50:D50"/>
+    <mergeCell ref="A145:D145"/>
+    <mergeCell ref="A86:D86"/>
     <mergeCell ref="A104:D104"/>
     <mergeCell ref="A95:D95"/>
-    <mergeCell ref="A113:D113"/>
     <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A71:D71"/>
-    <mergeCell ref="A47:D47"/>
-    <mergeCell ref="A42:D42"/>
+    <mergeCell ref="A33:D33"/>
+    <mergeCell ref="A32:D32"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2596,7 +2816,7 @@
         </is>
       </c>
       <c r="B3" s="21">
-        <f>80</f>
+        <f>91</f>
         <v/>
       </c>
     </row>
@@ -2607,7 +2827,7 @@
         </is>
       </c>
       <c r="B4" s="21">
-        <f>COUNTIF('7-Day Challenge Tracker'!D5:D131,TRUE)</f>
+        <f>COUNTIF('7-Day Challenge Tracker'!D5:D142,TRUE)</f>
         <v/>
       </c>
     </row>
@@ -2618,7 +2838,7 @@
         </is>
       </c>
       <c r="B5" s="21">
-        <f>80-COUNTIF('7-Day Challenge Tracker'!D5:D131,TRUE)</f>
+        <f>91-COUNTIF('7-Day Challenge Tracker'!D5:D142,TRUE)</f>
         <v/>
       </c>
     </row>
@@ -2629,7 +2849,7 @@
         </is>
       </c>
       <c r="B6" s="21">
-        <f>ROUND(COUNTIF('7-Day Challenge Tracker'!D5:D131,TRUE)/80*100,1)&amp;"%"</f>
+        <f>ROUND(COUNTIF('7-Day Challenge Tracker'!D5:D142,TRUE)/91*100,1)&amp;"%"</f>
         <v/>
       </c>
     </row>
@@ -2660,7 +2880,7 @@
       </c>
       <c r="B10" s="24" t="inlineStr">
         <is>
-          <t>9 items</t>
+          <t>11 items</t>
         </is>
       </c>
     </row>
@@ -2672,7 +2892,7 @@
       </c>
       <c r="B11" s="24" t="inlineStr">
         <is>
-          <t>10 items</t>
+          <t>12 items</t>
         </is>
       </c>
     </row>
@@ -2684,7 +2904,7 @@
       </c>
       <c r="B12" s="24" t="inlineStr">
         <is>
-          <t>10 items</t>
+          <t>12 items</t>
         </is>
       </c>
     </row>
@@ -2696,7 +2916,7 @@
       </c>
       <c r="B13" s="24" t="inlineStr">
         <is>
-          <t>10 items</t>
+          <t>12 items</t>
         </is>
       </c>
     </row>
@@ -2720,7 +2940,7 @@
       </c>
       <c r="B15" s="24" t="inlineStr">
         <is>
-          <t>11 items</t>
+          <t>14 items</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add videos to every challenge day (Days 0, 5, 7 were missing)
- Day 0: CC-003 preview (Master 95% of Claude Code) as watch-first intro
- Day 5: CC-002 (Build ANYTHING with Claude Code) for RAG context
- Day 7: CC-004 (Self-Healing Production Systems) for capstone patterns
All 8 days now have at least 1 video. 94 total items. Tracker updated.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Progress Tracker Template.xlsx
+++ b/Progress Tracker Template.xlsx
@@ -588,7 +588,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D145"/>
+  <dimension ref="A1:D148"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -650,17 +650,17 @@
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>CH-000a</t>
+          <t>CC-003-preview</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Lesson</t>
+          <t>Video</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>📖 Challenge Rules &amp; How It Works</t>
+          <t>🎬 Master 95% of Claude Code (Watch First)</t>
         </is>
       </c>
       <c r="D7" s="8" t="b">
@@ -670,17 +670,17 @@
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>CH-000b</t>
+          <t>CH-000a</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>Resource</t>
+          <t>Lesson</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>📋 Download Your Progress Tracker</t>
+          <t>📖 Challenge Rules &amp; How It Works</t>
         </is>
       </c>
       <c r="D8" s="8" t="b">
@@ -690,17 +690,17 @@
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>CH-000c</t>
+          <t>CH-000b</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Action</t>
+          <t>Resource</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>📢 Meet Your Fellow Builders</t>
+          <t>📋 Download Your Progress Tracker</t>
         </is>
       </c>
       <c r="D9" s="8" t="b">
@@ -710,118 +710,118 @@
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
+          <t>CH-000c</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>📢 Meet Your Fellow Builders</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
           <t>CH-000d</t>
         </is>
       </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>Lesson</t>
-        </is>
-      </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
         <is>
           <t>📖 Prerequisites &amp; Setup Checklist</t>
         </is>
       </c>
-      <c r="D10" s="8" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="inlineStr">
+      <c r="D11" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">  Rewards &amp; Recognition</t>
         </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>CH-000e</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>Lesson</t>
-        </is>
-      </c>
-      <c r="C12" s="7" t="inlineStr">
-        <is>
-          <t>📖 What You Unlock by Finishing</t>
-        </is>
-      </c>
-      <c r="D12" s="8" t="b">
-        <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
+          <t>CH-000e</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>📖 What You Unlock by Finishing</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
           <t>CH-000f</t>
         </is>
       </c>
-      <c r="B13" s="6" t="inlineStr">
-        <is>
-          <t>Lesson</t>
-        </is>
-      </c>
-      <c r="C13" s="7" t="inlineStr">
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
         <is>
           <t>📖 Hall of Builders</t>
         </is>
       </c>
-      <c r="D13" s="8" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" ht="28" customHeight="1">
-      <c r="A15" s="9" t="inlineStr">
+      <c r="D14" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" ht="28" customHeight="1">
+      <c r="A16" s="9" t="inlineStr">
         <is>
           <t>Day 1: Setup &amp; Your First Project</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="5" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">  Learn</t>
         </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="6" t="inlineStr">
-        <is>
-          <t>CH-101</t>
-        </is>
-      </c>
-      <c r="B17" s="6" t="inlineStr">
-        <is>
-          <t>Lesson</t>
-        </is>
-      </c>
-      <c r="C17" s="7" t="inlineStr">
-        <is>
-          <t>📖 What is Claude Code?</t>
-        </is>
-      </c>
-      <c r="D17" s="8" t="b">
-        <v>0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>CC-NEW-01</t>
+          <t>CH-101</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>Video</t>
+          <t>Lesson</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>🎬 How I'd Teach a 10 Year Old</t>
+          <t>📖 What is Claude Code?</t>
         </is>
       </c>
       <c r="D18" s="8" t="b">
@@ -831,7 +831,7 @@
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>CC-NEW-02</t>
+          <t>CC-NEW-01</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
@@ -841,7 +841,7 @@
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>🎬 Zero to Your First CC Workflow</t>
+          <t>🎬 How I'd Teach a 10 Year Old</t>
         </is>
       </c>
       <c r="D19" s="8" t="b">
@@ -851,7 +851,7 @@
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>CH-102</t>
+          <t>CC-NEW-02</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr">
@@ -861,7 +861,7 @@
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>🎬 Installing &amp; Configuring Claude Code</t>
+          <t>🎬 Zero to Your First CC Workflow</t>
         </is>
       </c>
       <c r="D20" s="8" t="b">
@@ -871,202 +871,202 @@
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
+          <t>CH-102</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>Video</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>🎬 Installing &amp; Configuring Claude Code</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
           <t>CH-103</t>
         </is>
       </c>
-      <c r="B21" s="6" t="inlineStr">
-        <is>
-          <t>Lesson</t>
-        </is>
-      </c>
-      <c r="C21" s="7" t="inlineStr">
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
         <is>
           <t>📖 The Claude Code Build Loop</t>
         </is>
       </c>
-      <c r="D21" s="8" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="5" t="inlineStr">
+      <c r="D22" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">  Build</t>
         </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="6" t="inlineStr">
-        <is>
-          <t>CH-104</t>
-        </is>
-      </c>
-      <c r="B23" s="6" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="C23" s="7" t="inlineStr">
-        <is>
-          <t>🔨 Project: Build a CLI Task Manager</t>
-        </is>
-      </c>
-      <c r="D23" s="8" t="b">
-        <v>0</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
+          <t>CH-104</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>🔨 Project: Build a CLI Task Manager</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
           <t>CH-105</t>
         </is>
       </c>
-      <c r="B24" s="6" t="inlineStr">
+      <c r="B25" s="6" t="inlineStr">
         <is>
           <t>Build</t>
         </is>
       </c>
-      <c r="C24" s="7" t="inlineStr">
+      <c r="C25" s="7" t="inlineStr">
         <is>
           <t>🔨 Bonus Build: Personal Expense Tracker</t>
         </is>
       </c>
-      <c r="D24" s="8" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="5" t="inlineStr">
+      <c r="D25" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">  Reference</t>
         </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="6" t="inlineStr">
-        <is>
-          <t>CH-106</t>
-        </is>
-      </c>
-      <c r="B26" s="6" t="inlineStr">
-        <is>
-          <t>Resource</t>
-        </is>
-      </c>
-      <c r="C26" s="7" t="inlineStr">
-        <is>
-          <t>📋 Claude Code Cheat Sheet</t>
-        </is>
-      </c>
-      <c r="D26" s="8" t="b">
-        <v>0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
+          <t>CH-106</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>Resource</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>📋 Claude Code Cheat Sheet</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
           <t>CH-107</t>
         </is>
       </c>
-      <c r="B27" s="6" t="inlineStr">
-        <is>
-          <t>Lesson</t>
-        </is>
-      </c>
-      <c r="C27" s="7" t="inlineStr">
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="C28" s="7" t="inlineStr">
         <is>
           <t>📖 Troubleshooting: Common Day 1 Issues</t>
         </is>
       </c>
-      <c r="D27" s="8" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="5" t="inlineStr">
+      <c r="D28" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">  Checkpoint</t>
         </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="6" t="inlineStr">
-        <is>
-          <t>CH-108</t>
-        </is>
-      </c>
-      <c r="B29" s="6" t="inlineStr">
-        <is>
-          <t>Quiz</t>
-        </is>
-      </c>
-      <c r="C29" s="7" t="inlineStr">
-        <is>
-          <t>❓ Day 1 Knowledge Check</t>
-        </is>
-      </c>
-      <c r="D29" s="8" t="b">
-        <v>0</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
+          <t>CH-108</t>
+        </is>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>Quiz</t>
+        </is>
+      </c>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>❓ Day 1 Knowledge Check</t>
+        </is>
+      </c>
+      <c r="D30" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
           <t>CH-109</t>
         </is>
       </c>
-      <c r="B30" s="6" t="inlineStr">
+      <c r="B31" s="6" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="C30" s="7" t="inlineStr">
+      <c r="C31" s="7" t="inlineStr">
         <is>
           <t>📢 Share Your Day 1 Build</t>
         </is>
       </c>
-      <c r="D30" s="8" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" ht="28" customHeight="1">
-      <c r="A32" s="10" t="inlineStr">
+      <c r="D31" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" ht="28" customHeight="1">
+      <c r="A33" s="10" t="inlineStr">
         <is>
           <t>Day 2: AI-Powered Applications</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="5" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">  Learn</t>
         </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="6" t="inlineStr">
-        <is>
-          <t>CC-NEW-03</t>
-        </is>
-      </c>
-      <c r="B34" s="6" t="inlineStr">
-        <is>
-          <t>Video</t>
-        </is>
-      </c>
-      <c r="C34" s="7" t="inlineStr">
-        <is>
-          <t>🎬 Firecrawl - Scrape Anything</t>
-        </is>
-      </c>
-      <c r="D34" s="8" t="b">
-        <v>0</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>CC-NEW-04</t>
+          <t>CC-NEW-03</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
@@ -1076,7 +1076,7 @@
       </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>🎬 Nano Banana 2 + Claude Code</t>
+          <t>🎬 Firecrawl - Scrape Anything</t>
         </is>
       </c>
       <c r="D35" s="8" t="b">
@@ -1086,17 +1086,17 @@
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>CH-201</t>
+          <t>CC-NEW-04</t>
         </is>
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>Lesson</t>
+          <t>Video</t>
         </is>
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>📖 Working with AI APIs Through Claude Code</t>
+          <t>🎬 Nano Banana 2 + Claude Code</t>
         </is>
       </c>
       <c r="D36" s="8" t="b">
@@ -1106,7 +1106,7 @@
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>CH-202</t>
+          <t>CH-201</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
@@ -1116,7 +1116,7 @@
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>📖 Giving Claude Code Context That Matters</t>
+          <t>📖 Working with AI APIs Through Claude Code</t>
         </is>
       </c>
       <c r="D37" s="8" t="b">
@@ -1126,54 +1126,54 @@
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
+          <t>CH-202</t>
+        </is>
+      </c>
+      <c r="B38" s="6" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="C38" s="7" t="inlineStr">
+        <is>
+          <t>📖 Giving Claude Code Context That Matters</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
           <t>CH-203</t>
         </is>
       </c>
-      <c r="B38" s="6" t="inlineStr">
-        <is>
-          <t>Lesson</t>
-        </is>
-      </c>
-      <c r="C38" s="7" t="inlineStr">
+      <c r="B39" s="6" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="C39" s="7" t="inlineStr">
         <is>
           <t>📖 Iterative Building: Start Simple, Then Layer</t>
         </is>
       </c>
-      <c r="D38" s="8" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="5" t="inlineStr">
+      <c r="D39" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">  Build</t>
         </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="6" t="inlineStr">
-        <is>
-          <t>CH-204</t>
-        </is>
-      </c>
-      <c r="B40" s="6" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="C40" s="7" t="inlineStr">
-        <is>
-          <t>🔨 Project: AI Content Generator</t>
-        </is>
-      </c>
-      <c r="D40" s="8" t="b">
-        <v>0</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>CH-205</t>
+          <t>CH-204</t>
         </is>
       </c>
       <c r="B41" s="6" t="inlineStr">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>🔨 Alternate Build: Smart URL Summarizer</t>
+          <t>🔨 Project: AI Content Generator</t>
         </is>
       </c>
       <c r="D41" s="8" t="b">
@@ -1193,155 +1193,155 @@
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
+          <t>CH-205</t>
+        </is>
+      </c>
+      <c r="B42" s="6" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="C42" s="7" t="inlineStr">
+        <is>
+          <t>🔨 Alternate Build: Smart URL Summarizer</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="inlineStr">
+        <is>
           <t>CH-206</t>
         </is>
       </c>
-      <c r="B42" s="6" t="inlineStr">
+      <c r="B43" s="6" t="inlineStr">
         <is>
           <t>Build</t>
         </is>
       </c>
-      <c r="C42" s="7" t="inlineStr">
+      <c r="C43" s="7" t="inlineStr">
         <is>
           <t>🔨 Alternate Build: Data Analysis Assistant</t>
         </is>
       </c>
-      <c r="D42" s="8" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="5" t="inlineStr">
+      <c r="D43" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">  Go Deeper</t>
         </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="6" t="inlineStr">
-        <is>
-          <t>CH-207</t>
-        </is>
-      </c>
-      <c r="B44" s="6" t="inlineStr">
-        <is>
-          <t>Lesson</t>
-        </is>
-      </c>
-      <c r="C44" s="7" t="inlineStr">
-        <is>
-          <t>📖 Environment Variables &amp; API Key Security</t>
-        </is>
-      </c>
-      <c r="D44" s="8" t="b">
-        <v>0</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
+          <t>CH-207</t>
+        </is>
+      </c>
+      <c r="B45" s="6" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="C45" s="7" t="inlineStr">
+        <is>
+          <t>📖 Environment Variables &amp; API Key Security</t>
+        </is>
+      </c>
+      <c r="D45" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="6" t="inlineStr">
+        <is>
           <t>CH-208</t>
         </is>
       </c>
-      <c r="B45" s="6" t="inlineStr">
-        <is>
-          <t>Lesson</t>
-        </is>
-      </c>
-      <c r="C45" s="7" t="inlineStr">
+      <c r="B46" s="6" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="C46" s="7" t="inlineStr">
         <is>
           <t>📖 Adding Error Handling &amp; Loading States</t>
         </is>
       </c>
-      <c r="D45" s="8" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="5" t="inlineStr">
+      <c r="D46" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">  Checkpoint</t>
         </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="6" t="inlineStr">
-        <is>
-          <t>CH-209</t>
-        </is>
-      </c>
-      <c r="B47" s="6" t="inlineStr">
-        <is>
-          <t>Quiz</t>
-        </is>
-      </c>
-      <c r="C47" s="7" t="inlineStr">
-        <is>
-          <t>❓ Day 2 Knowledge Check</t>
-        </is>
-      </c>
-      <c r="D47" s="8" t="b">
-        <v>0</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
+          <t>CH-209</t>
+        </is>
+      </c>
+      <c r="B48" s="6" t="inlineStr">
+        <is>
+          <t>Quiz</t>
+        </is>
+      </c>
+      <c r="C48" s="7" t="inlineStr">
+        <is>
+          <t>❓ Day 2 Knowledge Check</t>
+        </is>
+      </c>
+      <c r="D48" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="6" t="inlineStr">
+        <is>
           <t>CH-210</t>
         </is>
       </c>
-      <c r="B48" s="6" t="inlineStr">
+      <c r="B49" s="6" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="C48" s="7" t="inlineStr">
+      <c r="C49" s="7" t="inlineStr">
         <is>
           <t>📢 Share Your Day 2 Build</t>
         </is>
       </c>
-      <c r="D48" s="8" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50" ht="28" customHeight="1">
-      <c r="A50" s="11" t="inlineStr">
+      <c r="D49" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" ht="28" customHeight="1">
+      <c r="A51" s="11" t="inlineStr">
         <is>
           <t>Day 3: Master Claude Code</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="5" t="inlineStr">
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">  Learn</t>
         </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="6" t="inlineStr">
-        <is>
-          <t>CC-NEW-05</t>
-        </is>
-      </c>
-      <c r="B52" s="6" t="inlineStr">
-        <is>
-          <t>Video</t>
-        </is>
-      </c>
-      <c r="C52" s="7" t="inlineStr">
-        <is>
-          <t>🎬 Claude Code Skills</t>
-        </is>
-      </c>
-      <c r="D52" s="8" t="b">
-        <v>0</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>CC-NEW-06</t>
+          <t>CC-NEW-05</t>
         </is>
       </c>
       <c r="B53" s="6" t="inlineStr">
@@ -1351,7 +1351,7 @@
       </c>
       <c r="C53" s="7" t="inlineStr">
         <is>
-          <t>🎬 Claude Code Skills Just Got Even Better</t>
+          <t>🎬 Claude Code Skills</t>
         </is>
       </c>
       <c r="D53" s="8" t="b">
@@ -1361,7 +1361,7 @@
     <row r="54">
       <c r="A54" s="6" t="inlineStr">
         <is>
-          <t>CC-003</t>
+          <t>CC-NEW-06</t>
         </is>
       </c>
       <c r="B54" s="6" t="inlineStr">
@@ -1371,7 +1371,7 @@
       </c>
       <c r="C54" s="7" t="inlineStr">
         <is>
-          <t>🎬 Master 95% of Claude Code</t>
+          <t>🎬 Claude Code Skills Just Got Even Better</t>
         </is>
       </c>
       <c r="D54" s="8" t="b">
@@ -1381,17 +1381,17 @@
     <row r="55">
       <c r="A55" s="6" t="inlineStr">
         <is>
-          <t>CH-301</t>
+          <t>CC-003</t>
         </is>
       </c>
       <c r="B55" s="6" t="inlineStr">
         <is>
-          <t>Lesson</t>
+          <t>Video</t>
         </is>
       </c>
       <c r="C55" s="7" t="inlineStr">
         <is>
-          <t>📖 CLAUDE.md: Your Project's Brain</t>
+          <t>🎬 Master 95% of Claude Code</t>
         </is>
       </c>
       <c r="D55" s="8" t="b">
@@ -1401,7 +1401,7 @@
     <row r="56">
       <c r="A56" s="6" t="inlineStr">
         <is>
-          <t>CH-302</t>
+          <t>CH-301</t>
         </is>
       </c>
       <c r="B56" s="6" t="inlineStr">
@@ -1411,7 +1411,7 @@
       </c>
       <c r="C56" s="7" t="inlineStr">
         <is>
-          <t>📖 Prompt Patterns That Work</t>
+          <t>📖 CLAUDE.md: Your Project's Brain</t>
         </is>
       </c>
       <c r="D56" s="8" t="b">
@@ -1421,202 +1421,202 @@
     <row r="57">
       <c r="A57" s="6" t="inlineStr">
         <is>
+          <t>CH-302</t>
+        </is>
+      </c>
+      <c r="B57" s="6" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="C57" s="7" t="inlineStr">
+        <is>
+          <t>📖 Prompt Patterns That Work</t>
+        </is>
+      </c>
+      <c r="D57" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="6" t="inlineStr">
+        <is>
           <t>CH-303</t>
         </is>
       </c>
-      <c r="B57" s="6" t="inlineStr">
-        <is>
-          <t>Lesson</t>
-        </is>
-      </c>
-      <c r="C57" s="7" t="inlineStr">
+      <c r="B58" s="6" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="C58" s="7" t="inlineStr">
         <is>
           <t>📖 Multi-File Projects &amp; Code Organization</t>
         </is>
       </c>
-      <c r="D57" s="8" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="5" t="inlineStr">
+      <c r="D58" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">  Build</t>
         </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="6" t="inlineStr">
-        <is>
-          <t>CH-304</t>
-        </is>
-      </c>
-      <c r="B59" s="6" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="C59" s="7" t="inlineStr">
-        <is>
-          <t>🔨 Project: Three Mini-Builds, Three Techniques</t>
-        </is>
-      </c>
-      <c r="D59" s="8" t="b">
-        <v>0</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="6" t="inlineStr">
         <is>
+          <t>CH-304</t>
+        </is>
+      </c>
+      <c r="B60" s="6" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="C60" s="7" t="inlineStr">
+        <is>
+          <t>🔨 Project: Three Mini-Builds, Three Techniques</t>
+        </is>
+      </c>
+      <c r="D60" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="6" t="inlineStr">
+        <is>
           <t>CH-305</t>
         </is>
       </c>
-      <c r="B60" s="6" t="inlineStr">
+      <c r="B61" s="6" t="inlineStr">
         <is>
           <t>Build</t>
         </is>
       </c>
-      <c r="C60" s="7" t="inlineStr">
+      <c r="C61" s="7" t="inlineStr">
         <is>
           <t>🔨 Create Your First CLAUDE.md</t>
         </is>
       </c>
-      <c r="D60" s="8" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="5" t="inlineStr">
+      <c r="D61" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">  Go Deeper</t>
         </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="6" t="inlineStr">
-        <is>
-          <t>CH-306</t>
-        </is>
-      </c>
-      <c r="B62" s="6" t="inlineStr">
-        <is>
-          <t>Lesson</t>
-        </is>
-      </c>
-      <c r="C62" s="7" t="inlineStr">
-        <is>
-          <t>📖 Git Integration with Claude Code</t>
-        </is>
-      </c>
-      <c r="D62" s="8" t="b">
-        <v>0</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="6" t="inlineStr">
         <is>
+          <t>CH-306</t>
+        </is>
+      </c>
+      <c r="B63" s="6" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="C63" s="7" t="inlineStr">
+        <is>
+          <t>📖 Git Integration with Claude Code</t>
+        </is>
+      </c>
+      <c r="D63" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="6" t="inlineStr">
+        <is>
           <t>CH-307</t>
         </is>
       </c>
-      <c r="B63" s="6" t="inlineStr">
-        <is>
-          <t>Lesson</t>
-        </is>
-      </c>
-      <c r="C63" s="7" t="inlineStr">
+      <c r="B64" s="6" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="C64" s="7" t="inlineStr">
         <is>
           <t>📖 Debugging with Claude Code</t>
         </is>
       </c>
-      <c r="D63" s="8" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="5" t="inlineStr">
+      <c r="D64" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">  Checkpoint</t>
         </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="6" t="inlineStr">
-        <is>
-          <t>CH-308</t>
-        </is>
-      </c>
-      <c r="B65" s="6" t="inlineStr">
-        <is>
-          <t>Quiz</t>
-        </is>
-      </c>
-      <c r="C65" s="7" t="inlineStr">
-        <is>
-          <t>❓ Day 3 Knowledge Check</t>
-        </is>
-      </c>
-      <c r="D65" s="8" t="b">
-        <v>0</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="6" t="inlineStr">
         <is>
+          <t>CH-308</t>
+        </is>
+      </c>
+      <c r="B66" s="6" t="inlineStr">
+        <is>
+          <t>Quiz</t>
+        </is>
+      </c>
+      <c r="C66" s="7" t="inlineStr">
+        <is>
+          <t>❓ Day 3 Knowledge Check</t>
+        </is>
+      </c>
+      <c r="D66" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="6" t="inlineStr">
+        <is>
           <t>CH-309</t>
         </is>
       </c>
-      <c r="B66" s="6" t="inlineStr">
+      <c r="B67" s="6" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="C66" s="7" t="inlineStr">
+      <c r="C67" s="7" t="inlineStr">
         <is>
           <t>📢 Share Your Day 3 Builds</t>
         </is>
       </c>
-      <c r="D66" s="8" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="68" ht="28" customHeight="1">
-      <c r="A68" s="12" t="inlineStr">
+      <c r="D67" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" ht="28" customHeight="1">
+      <c r="A69" s="12" t="inlineStr">
         <is>
           <t>Day 4: Full-Stack Web Applications</t>
         </is>
       </c>
     </row>
-    <row r="69">
-      <c r="A69" s="5" t="inlineStr">
+    <row r="70">
+      <c r="A70" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">  Learn</t>
         </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="6" t="inlineStr">
-        <is>
-          <t>CC-NEW-07</t>
-        </is>
-      </c>
-      <c r="B70" s="6" t="inlineStr">
-        <is>
-          <t>Video</t>
-        </is>
-      </c>
-      <c r="C70" s="7" t="inlineStr">
-        <is>
-          <t>🎬 Website Building 5 Hacks</t>
-        </is>
-      </c>
-      <c r="D70" s="8" t="b">
-        <v>0</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>CC-NEW-08</t>
+          <t>CC-NEW-07</t>
         </is>
       </c>
       <c r="B71" s="6" t="inlineStr">
@@ -1626,7 +1626,7 @@
       </c>
       <c r="C71" s="7" t="inlineStr">
         <is>
-          <t>🎬 CC + Trigger.dev</t>
+          <t>🎬 Website Building 5 Hacks</t>
         </is>
       </c>
       <c r="D71" s="8" t="b">
@@ -1636,17 +1636,17 @@
     <row r="72">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>CH-401</t>
+          <t>CC-NEW-08</t>
         </is>
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>Lesson</t>
+          <t>Video</t>
         </is>
       </c>
       <c r="C72" s="7" t="inlineStr">
         <is>
-          <t>📖 Claude Code for Full-Stack Development</t>
+          <t>🎬 CC + Trigger.dev</t>
         </is>
       </c>
       <c r="D72" s="8" t="b">
@@ -1656,7 +1656,7 @@
     <row r="73">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>CH-402</t>
+          <t>CH-401</t>
         </is>
       </c>
       <c r="B73" s="6" t="inlineStr">
@@ -1666,7 +1666,7 @@
       </c>
       <c r="C73" s="7" t="inlineStr">
         <is>
-          <t>📖 The Product Spec Approach</t>
+          <t>📖 Claude Code for Full-Stack Development</t>
         </is>
       </c>
       <c r="D73" s="8" t="b">
@@ -1676,54 +1676,54 @@
     <row r="74">
       <c r="A74" s="6" t="inlineStr">
         <is>
+          <t>CH-402</t>
+        </is>
+      </c>
+      <c r="B74" s="6" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="C74" s="7" t="inlineStr">
+        <is>
+          <t>📖 The Product Spec Approach</t>
+        </is>
+      </c>
+      <c r="D74" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="6" t="inlineStr">
+        <is>
           <t>CH-403</t>
         </is>
       </c>
-      <c r="B74" s="6" t="inlineStr">
-        <is>
-          <t>Lesson</t>
-        </is>
-      </c>
-      <c r="C74" s="7" t="inlineStr">
+      <c r="B75" s="6" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="C75" s="7" t="inlineStr">
         <is>
           <t>📖 Databases with Claude Code</t>
         </is>
       </c>
-      <c r="D74" s="8" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="5" t="inlineStr">
+      <c r="D75" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">  Build</t>
         </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="6" t="inlineStr">
-        <is>
-          <t>CH-404</t>
-        </is>
-      </c>
-      <c r="B76" s="6" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="C76" s="7" t="inlineStr">
-        <is>
-          <t>🔨 Project: Build a Full-Stack Dashboard App</t>
-        </is>
-      </c>
-      <c r="D76" s="8" t="b">
-        <v>0</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="6" t="inlineStr">
         <is>
-          <t>CH-405</t>
+          <t>CH-404</t>
         </is>
       </c>
       <c r="B77" s="6" t="inlineStr">
@@ -1733,7 +1733,7 @@
       </c>
       <c r="C77" s="7" t="inlineStr">
         <is>
-          <t>🔨 Alternate Build: SaaS Landing Page with Auth</t>
+          <t>🔨 Project: Build a Full-Stack Dashboard App</t>
         </is>
       </c>
       <c r="D77" s="8" t="b">
@@ -1743,165 +1743,165 @@
     <row r="78">
       <c r="A78" s="6" t="inlineStr">
         <is>
+          <t>CH-405</t>
+        </is>
+      </c>
+      <c r="B78" s="6" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="C78" s="7" t="inlineStr">
+        <is>
+          <t>🔨 Alternate Build: SaaS Landing Page with Auth</t>
+        </is>
+      </c>
+      <c r="D78" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="6" t="inlineStr">
+        <is>
           <t>CH-406</t>
         </is>
       </c>
-      <c r="B78" s="6" t="inlineStr">
+      <c r="B79" s="6" t="inlineStr">
         <is>
           <t>Build</t>
         </is>
       </c>
-      <c r="C78" s="7" t="inlineStr">
+      <c r="C79" s="7" t="inlineStr">
         <is>
           <t>🔨 Alternate Build: API with Documentation</t>
         </is>
       </c>
-      <c r="D78" s="8" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" s="5" t="inlineStr">
+      <c r="D79" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">  Go Deeper</t>
         </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" s="6" t="inlineStr">
-        <is>
-          <t>CH-407</t>
-        </is>
-      </c>
-      <c r="B80" s="6" t="inlineStr">
-        <is>
-          <t>Lesson</t>
-        </is>
-      </c>
-      <c r="C80" s="7" t="inlineStr">
-        <is>
-          <t>📖 Deploying Your App to Vercel</t>
-        </is>
-      </c>
-      <c r="D80" s="8" t="b">
-        <v>0</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="6" t="inlineStr">
         <is>
+          <t>CH-407</t>
+        </is>
+      </c>
+      <c r="B81" s="6" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="C81" s="7" t="inlineStr">
+        <is>
+          <t>📖 Deploying Your App to Vercel</t>
+        </is>
+      </c>
+      <c r="D81" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="6" t="inlineStr">
+        <is>
           <t>CH-408</t>
         </is>
       </c>
-      <c r="B81" s="6" t="inlineStr">
-        <is>
-          <t>Lesson</t>
-        </is>
-      </c>
-      <c r="C81" s="7" t="inlineStr">
+      <c r="B82" s="6" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="C82" s="7" t="inlineStr">
         <is>
           <t>📖 Adding Real-Time Features</t>
         </is>
       </c>
-      <c r="D81" s="8" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" s="5" t="inlineStr">
+      <c r="D82" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">  Checkpoint</t>
         </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" s="6" t="inlineStr">
-        <is>
-          <t>CH-409</t>
-        </is>
-      </c>
-      <c r="B83" s="6" t="inlineStr">
-        <is>
-          <t>Quiz</t>
-        </is>
-      </c>
-      <c r="C83" s="7" t="inlineStr">
-        <is>
-          <t>❓ Day 4 Knowledge Check</t>
-        </is>
-      </c>
-      <c r="D83" s="8" t="b">
-        <v>0</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="6" t="inlineStr">
         <is>
+          <t>CH-409</t>
+        </is>
+      </c>
+      <c r="B84" s="6" t="inlineStr">
+        <is>
+          <t>Quiz</t>
+        </is>
+      </c>
+      <c r="C84" s="7" t="inlineStr">
+        <is>
+          <t>❓ Day 4 Knowledge Check</t>
+        </is>
+      </c>
+      <c r="D84" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="6" t="inlineStr">
+        <is>
           <t>CH-410</t>
         </is>
       </c>
-      <c r="B84" s="6" t="inlineStr">
+      <c r="B85" s="6" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="C84" s="7" t="inlineStr">
+      <c r="C85" s="7" t="inlineStr">
         <is>
           <t>📢 Share Your Day 4 Build</t>
         </is>
       </c>
-      <c r="D84" s="8" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="86" ht="28" customHeight="1">
-      <c r="A86" s="13" t="inlineStr">
+      <c r="D85" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87" ht="28" customHeight="1">
+      <c r="A87" s="13" t="inlineStr">
         <is>
           <t>Day 5: RAG &amp; AI Agent Systems</t>
         </is>
       </c>
     </row>
-    <row r="87">
-      <c r="A87" s="5" t="inlineStr">
+    <row r="88">
+      <c r="A88" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">  Learn</t>
         </is>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" s="6" t="inlineStr">
-        <is>
-          <t>CH-501</t>
-        </is>
-      </c>
-      <c r="B88" s="6" t="inlineStr">
-        <is>
-          <t>Lesson</t>
-        </is>
-      </c>
-      <c r="C88" s="7" t="inlineStr">
-        <is>
-          <t>📖 What is RAG and Why Every Business Wants It</t>
-        </is>
-      </c>
-      <c r="D88" s="8" t="b">
-        <v>0</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="6" t="inlineStr">
         <is>
-          <t>CH-502</t>
+          <t>CC-002-rag</t>
         </is>
       </c>
       <c r="B89" s="6" t="inlineStr">
         <is>
-          <t>Lesson</t>
+          <t>Video</t>
         </is>
       </c>
       <c r="C89" s="7" t="inlineStr">
         <is>
-          <t>📖 The RAG Pipeline: How It Works</t>
+          <t>🎬 Build ANYTHING with Claude Code</t>
         </is>
       </c>
       <c r="D89" s="8" t="b">
@@ -1911,7 +1911,7 @@
     <row r="90">
       <c r="A90" s="6" t="inlineStr">
         <is>
-          <t>CH-503</t>
+          <t>CH-501</t>
         </is>
       </c>
       <c r="B90" s="6" t="inlineStr">
@@ -1921,7 +1921,7 @@
       </c>
       <c r="C90" s="7" t="inlineStr">
         <is>
-          <t>📖 Choosing a Vector Database</t>
+          <t>📖 What is RAG and Why Every Business Wants It</t>
         </is>
       </c>
       <c r="D90" s="8" t="b">
@@ -1929,26 +1929,39 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Build</t>
-        </is>
+      <c r="A91" s="6" t="inlineStr">
+        <is>
+          <t>CH-502</t>
+        </is>
+      </c>
+      <c r="B91" s="6" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="C91" s="7" t="inlineStr">
+        <is>
+          <t>📖 The RAG Pipeline: How It Works</t>
+        </is>
+      </c>
+      <c r="D91" s="8" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="6" t="inlineStr">
         <is>
-          <t>CH-504</t>
+          <t>CH-503</t>
         </is>
       </c>
       <c r="B92" s="6" t="inlineStr">
         <is>
-          <t>Build</t>
+          <t>Lesson</t>
         </is>
       </c>
       <c r="C92" s="7" t="inlineStr">
         <is>
-          <t>🔨 Project: Chat With Your Documents</t>
+          <t>📖 Choosing a Vector Database</t>
         </is>
       </c>
       <c r="D92" s="8" t="b">
@@ -1956,29 +1969,16 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="6" t="inlineStr">
-        <is>
-          <t>CH-505</t>
-        </is>
-      </c>
-      <c r="B93" s="6" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="C93" s="7" t="inlineStr">
-        <is>
-          <t>🔨 Alternate Build: Research Assistant Agent</t>
-        </is>
-      </c>
-      <c r="D93" s="8" t="b">
-        <v>0</v>
+      <c r="A93" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Build</t>
+        </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="6" t="inlineStr">
         <is>
-          <t>CH-506</t>
+          <t>CH-504</t>
         </is>
       </c>
       <c r="B94" s="6" t="inlineStr">
@@ -1988,7 +1988,7 @@
       </c>
       <c r="C94" s="7" t="inlineStr">
         <is>
-          <t>🔨 Alternate Build: Q&amp;A Bot for Knowledge Base</t>
+          <t>🔨 Project: Chat With Your Documents</t>
         </is>
       </c>
       <c r="D94" s="8" t="b">
@@ -1996,26 +1996,39 @@
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Go Deeper</t>
-        </is>
+      <c r="A95" s="6" t="inlineStr">
+        <is>
+          <t>CH-505</t>
+        </is>
+      </c>
+      <c r="B95" s="6" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="C95" s="7" t="inlineStr">
+        <is>
+          <t>🔨 Alternate Build: Research Assistant Agent</t>
+        </is>
+      </c>
+      <c r="D95" s="8" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="6" t="inlineStr">
         <is>
-          <t>CH-507</t>
+          <t>CH-506</t>
         </is>
       </c>
       <c r="B96" s="6" t="inlineStr">
         <is>
-          <t>Lesson</t>
+          <t>Build</t>
         </is>
       </c>
       <c r="C96" s="7" t="inlineStr">
         <is>
-          <t>📖 Chunking Strategies That Matter</t>
+          <t>🔨 Alternate Build: Q&amp;A Bot for Knowledge Base</t>
         </is>
       </c>
       <c r="D96" s="8" t="b">
@@ -2023,29 +2036,16 @@
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="6" t="inlineStr">
-        <is>
-          <t>CH-508</t>
-        </is>
-      </c>
-      <c r="B97" s="6" t="inlineStr">
-        <is>
-          <t>Lesson</t>
-        </is>
-      </c>
-      <c r="C97" s="7" t="inlineStr">
-        <is>
-          <t>📖 Adding Memory to Your AI</t>
-        </is>
-      </c>
-      <c r="D97" s="8" t="b">
-        <v>0</v>
+      <c r="A97" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Go Deeper</t>
+        </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="6" t="inlineStr">
         <is>
-          <t>CH-509</t>
+          <t>CH-507</t>
         </is>
       </c>
       <c r="B98" s="6" t="inlineStr">
@@ -2055,7 +2055,7 @@
       </c>
       <c r="C98" s="7" t="inlineStr">
         <is>
-          <t>📖 Evaluating RAG Quality</t>
+          <t>📖 Chunking Strategies That Matter</t>
         </is>
       </c>
       <c r="D98" s="8" t="b">
@@ -2063,110 +2063,110 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Checkpoint</t>
-        </is>
+      <c r="A99" s="6" t="inlineStr">
+        <is>
+          <t>CH-508</t>
+        </is>
+      </c>
+      <c r="B99" s="6" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="C99" s="7" t="inlineStr">
+        <is>
+          <t>📖 Adding Memory to Your AI</t>
+        </is>
+      </c>
+      <c r="D99" s="8" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="6" t="inlineStr">
         <is>
+          <t>CH-509</t>
+        </is>
+      </c>
+      <c r="B100" s="6" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="C100" s="7" t="inlineStr">
+        <is>
+          <t>📖 Evaluating RAG Quality</t>
+        </is>
+      </c>
+      <c r="D100" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Checkpoint</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="6" t="inlineStr">
+        <is>
           <t>CH-510</t>
         </is>
       </c>
-      <c r="B100" s="6" t="inlineStr">
+      <c r="B102" s="6" t="inlineStr">
         <is>
           <t>Quiz</t>
         </is>
       </c>
-      <c r="C100" s="7" t="inlineStr">
+      <c r="C102" s="7" t="inlineStr">
         <is>
           <t>❓ Day 5 Knowledge Check</t>
         </is>
       </c>
-      <c r="D100" s="8" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" s="6" t="inlineStr">
+      <c r="D102" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="6" t="inlineStr">
         <is>
           <t>CH-511</t>
         </is>
       </c>
-      <c r="B101" s="6" t="inlineStr">
+      <c r="B103" s="6" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="C101" s="7" t="inlineStr">
+      <c r="C103" s="7" t="inlineStr">
         <is>
           <t>📢 Share Your Day 5 Build</t>
         </is>
       </c>
-      <c r="D101" s="8" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="103" ht="28" customHeight="1">
-      <c r="A103" s="14" t="inlineStr">
+      <c r="D103" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="105" ht="28" customHeight="1">
+      <c r="A105" s="14" t="inlineStr">
         <is>
           <t>Day 6: Complex Multi-Component Projects</t>
         </is>
       </c>
     </row>
-    <row r="104">
-      <c r="A104" s="5" t="inlineStr">
+    <row r="106">
+      <c r="A106" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">  Learn</t>
         </is>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" s="6" t="inlineStr">
-        <is>
-          <t>CC-NEW-09</t>
-        </is>
-      </c>
-      <c r="B105" s="6" t="inlineStr">
-        <is>
-          <t>Video</t>
-        </is>
-      </c>
-      <c r="C105" s="7" t="inlineStr">
-        <is>
-          <t>🎬 Claude Code Executive Assistant</t>
-        </is>
-      </c>
-      <c r="D105" s="8" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" s="6" t="inlineStr">
-        <is>
-          <t>CC-NEW-10</t>
-        </is>
-      </c>
-      <c r="B106" s="6" t="inlineStr">
-        <is>
-          <t>Video</t>
-        </is>
-      </c>
-      <c r="C106" s="7" t="inlineStr">
-        <is>
-          <t>🎬 Watch My AI Agents Work in Real Time</t>
-        </is>
-      </c>
-      <c r="D106" s="8" t="b">
-        <v>0</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="6" t="inlineStr">
         <is>
-          <t>CC-NEW-11</t>
+          <t>CC-NEW-09</t>
         </is>
       </c>
       <c r="B107" s="6" t="inlineStr">
@@ -2176,7 +2176,7 @@
       </c>
       <c r="C107" s="7" t="inlineStr">
         <is>
-          <t>🎬 Claude Code Remote Control</t>
+          <t>🎬 Claude Code Executive Assistant</t>
         </is>
       </c>
       <c r="D107" s="8" t="b">
@@ -2186,17 +2186,17 @@
     <row r="108">
       <c r="A108" s="6" t="inlineStr">
         <is>
-          <t>CH-601</t>
+          <t>CC-NEW-10</t>
         </is>
       </c>
       <c r="B108" s="6" t="inlineStr">
         <is>
-          <t>Lesson</t>
+          <t>Video</t>
         </is>
       </c>
       <c r="C108" s="7" t="inlineStr">
         <is>
-          <t>📖 Thinking in Systems, Not Scripts</t>
+          <t>🎬 Watch My AI Agents Work in Real Time</t>
         </is>
       </c>
       <c r="D108" s="8" t="b">
@@ -2206,17 +2206,17 @@
     <row r="109">
       <c r="A109" s="6" t="inlineStr">
         <is>
-          <t>CH-602</t>
+          <t>CC-NEW-11</t>
         </is>
       </c>
       <c r="B109" s="6" t="inlineStr">
         <is>
-          <t>Lesson</t>
+          <t>Video</t>
         </is>
       </c>
       <c r="C109" s="7" t="inlineStr">
         <is>
-          <t>📖 API Design Patterns</t>
+          <t>🎬 Claude Code Remote Control</t>
         </is>
       </c>
       <c r="D109" s="8" t="b">
@@ -2226,7 +2226,7 @@
     <row r="110">
       <c r="A110" s="6" t="inlineStr">
         <is>
-          <t>CH-603</t>
+          <t>CH-601</t>
         </is>
       </c>
       <c r="B110" s="6" t="inlineStr">
@@ -2236,7 +2236,7 @@
       </c>
       <c r="C110" s="7" t="inlineStr">
         <is>
-          <t>📖 Working with External Services</t>
+          <t>📖 Thinking in Systems, Not Scripts</t>
         </is>
       </c>
       <c r="D110" s="8" t="b">
@@ -2244,26 +2244,39 @@
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Build</t>
-        </is>
+      <c r="A111" s="6" t="inlineStr">
+        <is>
+          <t>CH-602</t>
+        </is>
+      </c>
+      <c r="B111" s="6" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="C111" s="7" t="inlineStr">
+        <is>
+          <t>📖 API Design Patterns</t>
+        </is>
+      </c>
+      <c r="D111" s="8" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="6" t="inlineStr">
         <is>
-          <t>CH-604</t>
+          <t>CH-603</t>
         </is>
       </c>
       <c r="B112" s="6" t="inlineStr">
         <is>
-          <t>Build</t>
+          <t>Lesson</t>
         </is>
       </c>
       <c r="C112" s="7" t="inlineStr">
         <is>
-          <t>🔨 Project: Multi-Service Application</t>
+          <t>📖 Working with External Services</t>
         </is>
       </c>
       <c r="D112" s="8" t="b">
@@ -2271,29 +2284,16 @@
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="6" t="inlineStr">
-        <is>
-          <t>CH-605</t>
-        </is>
-      </c>
-      <c r="B113" s="6" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="C113" s="7" t="inlineStr">
-        <is>
-          <t>🔨 Alternate Build: Slack Bot</t>
-        </is>
-      </c>
-      <c r="D113" s="8" t="b">
-        <v>0</v>
+      <c r="A113" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Build</t>
+        </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="6" t="inlineStr">
         <is>
-          <t>CH-606</t>
+          <t>CH-604</t>
         </is>
       </c>
       <c r="B114" s="6" t="inlineStr">
@@ -2303,7 +2303,7 @@
       </c>
       <c r="C114" s="7" t="inlineStr">
         <is>
-          <t>🔨 Alternate Build: Chrome Extension</t>
+          <t>🔨 Project: Multi-Service Application</t>
         </is>
       </c>
       <c r="D114" s="8" t="b">
@@ -2311,26 +2311,39 @@
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Go Deeper</t>
-        </is>
+      <c r="A115" s="6" t="inlineStr">
+        <is>
+          <t>CH-605</t>
+        </is>
+      </c>
+      <c r="B115" s="6" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="C115" s="7" t="inlineStr">
+        <is>
+          <t>🔨 Alternate Build: Slack Bot</t>
+        </is>
+      </c>
+      <c r="D115" s="8" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="6" t="inlineStr">
         <is>
-          <t>CH-607</t>
+          <t>CH-606</t>
         </is>
       </c>
       <c r="B116" s="6" t="inlineStr">
         <is>
-          <t>Lesson</t>
+          <t>Build</t>
         </is>
       </c>
       <c r="C116" s="7" t="inlineStr">
         <is>
-          <t>📖 Testing Your Code with Claude Code</t>
+          <t>🔨 Alternate Build: Chrome Extension</t>
         </is>
       </c>
       <c r="D116" s="8" t="b">
@@ -2338,29 +2351,16 @@
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="6" t="inlineStr">
-        <is>
-          <t>CH-608</t>
-        </is>
-      </c>
-      <c r="B117" s="6" t="inlineStr">
-        <is>
-          <t>Lesson</t>
-        </is>
-      </c>
-      <c r="C117" s="7" t="inlineStr">
-        <is>
-          <t>📖 Error Handling &amp; Logging</t>
-        </is>
-      </c>
-      <c r="D117" s="8" t="b">
-        <v>0</v>
+      <c r="A117" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Go Deeper</t>
+        </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="6" t="inlineStr">
         <is>
-          <t>CH-609</t>
+          <t>CH-607</t>
         </is>
       </c>
       <c r="B118" s="6" t="inlineStr">
@@ -2370,7 +2370,7 @@
       </c>
       <c r="C118" s="7" t="inlineStr">
         <is>
-          <t>📖 Rate Limiting &amp; Security Basics</t>
+          <t>📖 Testing Your Code with Claude Code</t>
         </is>
       </c>
       <c r="D118" s="8" t="b">
@@ -2378,120 +2378,120 @@
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Checkpoint</t>
-        </is>
+      <c r="A119" s="6" t="inlineStr">
+        <is>
+          <t>CH-608</t>
+        </is>
+      </c>
+      <c r="B119" s="6" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="C119" s="7" t="inlineStr">
+        <is>
+          <t>📖 Error Handling &amp; Logging</t>
+        </is>
+      </c>
+      <c r="D119" s="8" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="6" t="inlineStr">
         <is>
+          <t>CH-609</t>
+        </is>
+      </c>
+      <c r="B120" s="6" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="C120" s="7" t="inlineStr">
+        <is>
+          <t>📖 Rate Limiting &amp; Security Basics</t>
+        </is>
+      </c>
+      <c r="D120" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Checkpoint</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="6" t="inlineStr">
+        <is>
           <t>CH-610</t>
         </is>
       </c>
-      <c r="B120" s="6" t="inlineStr">
+      <c r="B122" s="6" t="inlineStr">
         <is>
           <t>Quiz</t>
         </is>
       </c>
-      <c r="C120" s="7" t="inlineStr">
+      <c r="C122" s="7" t="inlineStr">
         <is>
           <t>❓ Day 6 Knowledge Check</t>
         </is>
       </c>
-      <c r="D120" s="8" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" s="6" t="inlineStr">
+      <c r="D122" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="6" t="inlineStr">
         <is>
           <t>CH-611</t>
         </is>
       </c>
-      <c r="B121" s="6" t="inlineStr">
+      <c r="B123" s="6" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="C121" s="7" t="inlineStr">
+      <c r="C123" s="7" t="inlineStr">
         <is>
           <t>📢 Share Your Day 6 Build</t>
         </is>
       </c>
-      <c r="D121" s="8" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="123" ht="28" customHeight="1">
-      <c r="A123" s="15" t="inlineStr">
+      <c r="D123" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="125" ht="28" customHeight="1">
+      <c r="A125" s="15" t="inlineStr">
         <is>
           <t>Day 7: Production-Grade Capstone</t>
         </is>
       </c>
     </row>
-    <row r="124">
-      <c r="A124" s="5" t="inlineStr">
+    <row r="126">
+      <c r="A126" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">  Learn</t>
         </is>
-      </c>
-    </row>
-    <row r="125">
-      <c r="A125" s="6" t="inlineStr">
-        <is>
-          <t>CH-701</t>
-        </is>
-      </c>
-      <c r="B125" s="6" t="inlineStr">
-        <is>
-          <t>Lesson</t>
-        </is>
-      </c>
-      <c r="C125" s="7" t="inlineStr">
-        <is>
-          <t>📖 What Makes Something Production-Grade</t>
-        </is>
-      </c>
-      <c r="D125" s="8" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" s="6" t="inlineStr">
-        <is>
-          <t>CH-702</t>
-        </is>
-      </c>
-      <c r="B126" s="6" t="inlineStr">
-        <is>
-          <t>Lesson</t>
-        </is>
-      </c>
-      <c r="C126" s="7" t="inlineStr">
-        <is>
-          <t>📖 Documentation That Sells Your Work</t>
-        </is>
-      </c>
-      <c r="D126" s="8" t="b">
-        <v>0</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="6" t="inlineStr">
         <is>
-          <t>CH-703</t>
+          <t>CC-004-prod</t>
         </is>
       </c>
       <c r="B127" s="6" t="inlineStr">
         <is>
-          <t>Lesson</t>
+          <t>Video</t>
         </is>
       </c>
       <c r="C127" s="7" t="inlineStr">
         <is>
-          <t>📖 CI/CD and Automated Deployment</t>
+          <t>🎬 Self-Healing Production Systems</t>
         </is>
       </c>
       <c r="D127" s="8" t="b">
@@ -2499,26 +2499,39 @@
       </c>
     </row>
     <row r="128">
-      <c r="A128" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Build</t>
-        </is>
+      <c r="A128" s="6" t="inlineStr">
+        <is>
+          <t>CH-701</t>
+        </is>
+      </c>
+      <c r="B128" s="6" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="C128" s="7" t="inlineStr">
+        <is>
+          <t>📖 What Makes Something Production-Grade</t>
+        </is>
+      </c>
+      <c r="D128" s="8" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="6" t="inlineStr">
         <is>
-          <t>CH-704</t>
+          <t>CH-702</t>
         </is>
       </c>
       <c r="B129" s="6" t="inlineStr">
         <is>
-          <t>Build</t>
+          <t>Lesson</t>
         </is>
       </c>
       <c r="C129" s="7" t="inlineStr">
         <is>
-          <t>🔨 Capstone: Make Your Best Project Production-Ready</t>
+          <t>📖 Documentation That Sells Your Work</t>
         </is>
       </c>
       <c r="D129" s="8" t="b">
@@ -2528,64 +2541,64 @@
     <row r="130">
       <c r="A130" s="6" t="inlineStr">
         <is>
-          <t>CH-705</t>
+          <t>CH-703</t>
         </is>
       </c>
       <c r="B130" s="6" t="inlineStr">
         <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="C130" s="7" t="inlineStr">
+        <is>
+          <t>📖 CI/CD and Automated Deployment</t>
+        </is>
+      </c>
+      <c r="D130" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Build</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="6" t="inlineStr">
+        <is>
+          <t>CH-704</t>
+        </is>
+      </c>
+      <c r="B132" s="6" t="inlineStr">
+        <is>
           <t>Build</t>
         </is>
       </c>
-      <c r="C130" s="7" t="inlineStr">
-        <is>
-          <t>🔨 Add a Feature You've Been Wanting</t>
-        </is>
-      </c>
-      <c r="D130" s="8" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" s="6" t="inlineStr">
-        <is>
-          <t>CH-706</t>
-        </is>
-      </c>
-      <c r="B131" s="6" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="C131" s="7" t="inlineStr">
-        <is>
-          <t>🔨 Code Review: Ask Claude to Review Your Code</t>
-        </is>
-      </c>
-      <c r="D131" s="8" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="132">
-      <c r="A132" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Go Deeper</t>
-        </is>
+      <c r="C132" s="7" t="inlineStr">
+        <is>
+          <t>🔨 Capstone: Make Your Best Project Production-Ready</t>
+        </is>
+      </c>
+      <c r="D132" s="8" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="6" t="inlineStr">
         <is>
-          <t>CH-707</t>
+          <t>CH-705</t>
         </is>
       </c>
       <c r="B133" s="6" t="inlineStr">
         <is>
-          <t>Lesson</t>
+          <t>Build</t>
         </is>
       </c>
       <c r="C133" s="7" t="inlineStr">
         <is>
-          <t>📖 Performance Optimization</t>
+          <t>🔨 Add a Feature You've Been Wanting</t>
         </is>
       </c>
       <c r="D133" s="8" t="b">
@@ -2595,17 +2608,17 @@
     <row r="134">
       <c r="A134" s="6" t="inlineStr">
         <is>
-          <t>CH-708</t>
+          <t>CH-706</t>
         </is>
       </c>
       <c r="B134" s="6" t="inlineStr">
         <is>
-          <t>Lesson</t>
+          <t>Build</t>
         </is>
       </c>
       <c r="C134" s="7" t="inlineStr">
         <is>
-          <t>📖 Monitoring &amp; Health Checks</t>
+          <t>🔨 Code Review: Ask Claude to Review Your Code</t>
         </is>
       </c>
       <c r="D134" s="8" t="b">
@@ -2613,46 +2626,46 @@
       </c>
     </row>
     <row r="135">
-      <c r="A135" s="6" t="inlineStr">
-        <is>
-          <t>CH-709</t>
-        </is>
-      </c>
-      <c r="B135" s="6" t="inlineStr">
-        <is>
-          <t>Lesson</t>
-        </is>
-      </c>
-      <c r="C135" s="7" t="inlineStr">
-        <is>
-          <t>📖 Preparing for a Portfolio</t>
-        </is>
-      </c>
-      <c r="D135" s="8" t="b">
-        <v>0</v>
+      <c r="A135" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Go Deeper</t>
+        </is>
       </c>
     </row>
     <row r="136">
-      <c r="A136" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Challenge Complete</t>
-        </is>
+      <c r="A136" s="6" t="inlineStr">
+        <is>
+          <t>CH-707</t>
+        </is>
+      </c>
+      <c r="B136" s="6" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="C136" s="7" t="inlineStr">
+        <is>
+          <t>📖 Performance Optimization</t>
+        </is>
+      </c>
+      <c r="D136" s="8" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="6" t="inlineStr">
         <is>
-          <t>CH-710</t>
+          <t>CH-708</t>
         </is>
       </c>
       <c r="B137" s="6" t="inlineStr">
         <is>
-          <t>Quiz</t>
+          <t>Lesson</t>
         </is>
       </c>
       <c r="C137" s="7" t="inlineStr">
         <is>
-          <t>❓ Day 7 Knowledge Check (Final)</t>
+          <t>📖 Monitoring &amp; Health Checks</t>
         </is>
       </c>
       <c r="D137" s="8" t="b">
@@ -2662,17 +2675,17 @@
     <row r="138">
       <c r="A138" s="6" t="inlineStr">
         <is>
-          <t>CH-711</t>
+          <t>CH-709</t>
         </is>
       </c>
       <c r="B138" s="6" t="inlineStr">
         <is>
-          <t>Action</t>
+          <t>Lesson</t>
         </is>
       </c>
       <c r="C138" s="7" t="inlineStr">
         <is>
-          <t>📢 Submit Your Capstone</t>
+          <t>📖 Preparing for a Portfolio</t>
         </is>
       </c>
       <c r="D138" s="8" t="b">
@@ -2680,110 +2693,157 @@
       </c>
     </row>
     <row r="139">
-      <c r="A139" s="6" t="inlineStr">
-        <is>
-          <t>CH-712</t>
-        </is>
-      </c>
-      <c r="B139" s="6" t="inlineStr">
-        <is>
-          <t>Reward</t>
-        </is>
-      </c>
-      <c r="C139" s="7" t="inlineStr">
-        <is>
-          <t>🏆 Claim Your Challenge Rewards</t>
-        </is>
-      </c>
-      <c r="D139" s="8" t="b">
-        <v>0</v>
+      <c r="A139" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Challenge Complete</t>
+        </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="6" t="inlineStr">
         <is>
+          <t>CH-710</t>
+        </is>
+      </c>
+      <c r="B140" s="6" t="inlineStr">
+        <is>
+          <t>Quiz</t>
+        </is>
+      </c>
+      <c r="C140" s="7" t="inlineStr">
+        <is>
+          <t>❓ Day 7 Knowledge Check (Final)</t>
+        </is>
+      </c>
+      <c r="D140" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="6" t="inlineStr">
+        <is>
+          <t>CH-711</t>
+        </is>
+      </c>
+      <c r="B141" s="6" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="C141" s="7" t="inlineStr">
+        <is>
+          <t>📢 Submit Your Capstone</t>
+        </is>
+      </c>
+      <c r="D141" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="6" t="inlineStr">
+        <is>
+          <t>CH-712</t>
+        </is>
+      </c>
+      <c r="B142" s="6" t="inlineStr">
+        <is>
+          <t>Reward</t>
+        </is>
+      </c>
+      <c r="C142" s="7" t="inlineStr">
+        <is>
+          <t>🏆 Claim Your Challenge Rewards</t>
+        </is>
+      </c>
+      <c r="D142" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="6" t="inlineStr">
+        <is>
           <t>CH-713</t>
         </is>
       </c>
-      <c r="B140" s="6" t="inlineStr">
-        <is>
-          <t>Lesson</t>
-        </is>
-      </c>
-      <c r="C140" s="7" t="inlineStr">
+      <c r="B143" s="6" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="C143" s="7" t="inlineStr">
         <is>
           <t>📖 Your Path Forward</t>
         </is>
       </c>
-      <c r="D140" s="8" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="143">
-      <c r="A143" s="16" t="inlineStr">
+      <c r="D143" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="16" t="inlineStr">
         <is>
           <t>REWARD ELIGIBILITY</t>
         </is>
       </c>
     </row>
-    <row r="144" ht="35" customHeight="1">
-      <c r="A144" s="17">
-        <f>IF(AND(D23=TRUE,D40=TRUE,D59=TRUE,D76=TRUE,D92=TRUE,D112=TRUE,D129=TRUE),"🏆 Ready to Claim!","Keep building — complete the main build for each day")</f>
+    <row r="147" ht="35" customHeight="1">
+      <c r="A147" s="17">
+        <f>IF(AND(D24=TRUE,D41=TRUE,D60=TRUE,D77=TRUE,D94=TRUE,D114=TRUE,D132=TRUE),"🏆 Ready to Claim!","Keep building — complete the main build for each day")</f>
         <v/>
       </c>
     </row>
-    <row r="145">
-      <c r="A145" s="18" t="inlineStr">
-        <is>
-          <t>Main builds tracked: Day 1 (row 23), Day 2 (row 40), Day 3 (row 59), Day 4 (row 76), Day 5 (row 92), Day 6 (row 112), Day 7 (row 129)</t>
+    <row r="148">
+      <c r="A148" s="18" t="inlineStr">
+        <is>
+          <t>Main builds tracked: Day 1 (row 24), Day 2 (row 41), Day 3 (row 60), Day 4 (row 77), Day 5 (row 94), Day 6 (row 114), Day 7 (row 132)</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="43">
     <mergeCell ref="A5:D5"/>
-    <mergeCell ref="A144:D144"/>
-    <mergeCell ref="A22:D22"/>
-    <mergeCell ref="A91:D91"/>
-    <mergeCell ref="A43:D43"/>
-    <mergeCell ref="A28:D28"/>
-    <mergeCell ref="A115:D115"/>
-    <mergeCell ref="A68:D68"/>
-    <mergeCell ref="A111:D111"/>
-    <mergeCell ref="A58:D58"/>
-    <mergeCell ref="A143:D143"/>
-    <mergeCell ref="A39:D39"/>
-    <mergeCell ref="A15:D15"/>
-    <mergeCell ref="A64:D64"/>
-    <mergeCell ref="A82:D82"/>
+    <mergeCell ref="A17:D17"/>
+    <mergeCell ref="A23:D23"/>
+    <mergeCell ref="A126:D126"/>
+    <mergeCell ref="A106:D106"/>
+    <mergeCell ref="A97:D97"/>
+    <mergeCell ref="A135:D135"/>
+    <mergeCell ref="A131:D131"/>
+    <mergeCell ref="A62:D62"/>
+    <mergeCell ref="A147:D147"/>
+    <mergeCell ref="A29:D29"/>
+    <mergeCell ref="A52:D52"/>
+    <mergeCell ref="A125:D125"/>
+    <mergeCell ref="A121:D121"/>
+    <mergeCell ref="A117:D117"/>
+    <mergeCell ref="A93:D93"/>
+    <mergeCell ref="A44:D44"/>
+    <mergeCell ref="A40:D40"/>
+    <mergeCell ref="A34:D34"/>
+    <mergeCell ref="A83:D83"/>
+    <mergeCell ref="A148:D148"/>
+    <mergeCell ref="A59:D59"/>
     <mergeCell ref="A51:D51"/>
-    <mergeCell ref="A11:D11"/>
-    <mergeCell ref="A123:D123"/>
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A103:D103"/>
-    <mergeCell ref="A132:D132"/>
-    <mergeCell ref="A79:D79"/>
-    <mergeCell ref="A61:D61"/>
+    <mergeCell ref="A70:D70"/>
+    <mergeCell ref="A146:D146"/>
     <mergeCell ref="A6:D6"/>
-    <mergeCell ref="A119:D119"/>
+    <mergeCell ref="A88:D88"/>
     <mergeCell ref="A69:D69"/>
-    <mergeCell ref="A124:D124"/>
     <mergeCell ref="A87:D87"/>
-    <mergeCell ref="A25:D25"/>
-    <mergeCell ref="A128:D128"/>
+    <mergeCell ref="A65:D65"/>
     <mergeCell ref="A16:D16"/>
-    <mergeCell ref="A99:D99"/>
-    <mergeCell ref="A46:D46"/>
-    <mergeCell ref="A75:D75"/>
-    <mergeCell ref="A136:D136"/>
-    <mergeCell ref="A50:D50"/>
-    <mergeCell ref="A145:D145"/>
-    <mergeCell ref="A86:D86"/>
-    <mergeCell ref="A104:D104"/>
-    <mergeCell ref="A95:D95"/>
+    <mergeCell ref="A80:D80"/>
+    <mergeCell ref="A105:D105"/>
+    <mergeCell ref="A12:D12"/>
+    <mergeCell ref="A26:D26"/>
+    <mergeCell ref="A101:D101"/>
+    <mergeCell ref="A139:D139"/>
+    <mergeCell ref="A113:D113"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="A33:D33"/>
-    <mergeCell ref="A32:D32"/>
+    <mergeCell ref="A47:D47"/>
+    <mergeCell ref="A76:D76"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2816,7 +2876,7 @@
         </is>
       </c>
       <c r="B3" s="21">
-        <f>91</f>
+        <f>94</f>
         <v/>
       </c>
     </row>
@@ -2827,7 +2887,7 @@
         </is>
       </c>
       <c r="B4" s="21">
-        <f>COUNTIF('7-Day Challenge Tracker'!D5:D142,TRUE)</f>
+        <f>COUNTIF('7-Day Challenge Tracker'!D5:D145,TRUE)</f>
         <v/>
       </c>
     </row>
@@ -2838,7 +2898,7 @@
         </is>
       </c>
       <c r="B5" s="21">
-        <f>91-COUNTIF('7-Day Challenge Tracker'!D5:D142,TRUE)</f>
+        <f>94-COUNTIF('7-Day Challenge Tracker'!D5:D145,TRUE)</f>
         <v/>
       </c>
     </row>
@@ -2849,7 +2909,7 @@
         </is>
       </c>
       <c r="B6" s="21">
-        <f>ROUND(COUNTIF('7-Day Challenge Tracker'!D5:D142,TRUE)/91*100,1)&amp;"%"</f>
+        <f>ROUND(COUNTIF('7-Day Challenge Tracker'!D5:D145,TRUE)/94*100,1)&amp;"%"</f>
         <v/>
       </c>
     </row>
@@ -2868,7 +2928,7 @@
       </c>
       <c r="B9" s="24" t="inlineStr">
         <is>
-          <t>6 items</t>
+          <t>7 items (1 videos)</t>
         </is>
       </c>
     </row>
@@ -2880,7 +2940,7 @@
       </c>
       <c r="B10" s="24" t="inlineStr">
         <is>
-          <t>11 items</t>
+          <t>11 items (3 videos)</t>
         </is>
       </c>
     </row>
@@ -2892,7 +2952,7 @@
       </c>
       <c r="B11" s="24" t="inlineStr">
         <is>
-          <t>12 items</t>
+          <t>12 items (2 videos)</t>
         </is>
       </c>
     </row>
@@ -2904,7 +2964,7 @@
       </c>
       <c r="B12" s="24" t="inlineStr">
         <is>
-          <t>12 items</t>
+          <t>12 items (3 videos)</t>
         </is>
       </c>
     </row>
@@ -2916,7 +2976,7 @@
       </c>
       <c r="B13" s="24" t="inlineStr">
         <is>
-          <t>12 items</t>
+          <t>12 items (2 videos)</t>
         </is>
       </c>
     </row>
@@ -2928,7 +2988,7 @@
       </c>
       <c r="B14" s="24" t="inlineStr">
         <is>
-          <t>11 items</t>
+          <t>12 items (1 videos)</t>
         </is>
       </c>
     </row>
@@ -2940,7 +3000,7 @@
       </c>
       <c r="B15" s="24" t="inlineStr">
         <is>
-          <t>14 items</t>
+          <t>14 items (3 videos)</t>
         </is>
       </c>
     </row>
@@ -2952,7 +3012,7 @@
       </c>
       <c r="B16" s="24" t="inlineStr">
         <is>
-          <t>13 items</t>
+          <t>14 items (1 videos)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rewrite all challenge content from actual video transcripts
Transcribed all 8 YouTube videos and rewrote every description,
lesson, build instruction, quiz question, and Go Deeper section
to accurately reflect what Nate actually covers:
- Day 1: WAT framework, newsletter automation (Perplexity + Nano Banana + Gmail)
- Day 2: Firecrawl MCP server (scrape/map/crawl/extract)
- Day 3: Skills anatomy, progressive loading, 6-step framework, Skill Builder
- Day 4: Trigger.dev deployment, GitHub auto-deploy pipeline, dental lead generator
- Day 5: 5 website hacks (front-end skill, screenshot loop, site cloning, 21st.dev)
- Day 6: Scheduled tasks (desktop app) + Loop feature (cron create/list/delete)
- Day 7: Executive assistant (4 phases: Home, Life, Hands, Growth)

Updated progress tracker to match new item titles.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Progress Tracker Template.xlsx
+++ b/Progress Tracker Template.xlsx
@@ -645,7 +645,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="55" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
   </cols>
@@ -862,7 +862,7 @@
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>📖 The Describe → Generate → Review → Iterate Loop</t>
+          <t>📖 The WAT Framework &amp; How Claude Code Projects Work</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
@@ -894,7 +894,7 @@
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>🔨 Replicate Nate's Build from the Video</t>
+          <t>🔨 Build the Newsletter Automation from the Video</t>
         </is>
       </c>
       <c r="C16" s="8" t="inlineStr">
@@ -916,7 +916,7 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>🔨 Extend Your Build</t>
+          <t>🔨 Customize Your Newsletter</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
@@ -948,7 +948,7 @@
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>📖 Iteration Techniques from the Video</t>
+          <t>📖 Agentic vs Traditional Automation &amp; Value-Based Pricing</t>
         </is>
       </c>
       <c r="C19" s="8" t="inlineStr">
@@ -1098,7 +1098,7 @@
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>🔨 Set Up and Build with an MCP Server</t>
+          <t>🔨 Set Up Firecrawl MCP &amp; Scrape Your First Site</t>
         </is>
       </c>
       <c r="C29" s="8" t="inlineStr">
@@ -1120,7 +1120,7 @@
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>🔨 Build Something New with Your MCP Connection</t>
+          <t>🔨 Extract Structured Data from a Real Website</t>
         </is>
       </c>
       <c r="C30" s="8" t="inlineStr">
@@ -1152,7 +1152,7 @@
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t>📖 Exploring Other MCP Servers</t>
+          <t>📖 Running Parallel Agents &amp; Exploring Other MCP Servers</t>
         </is>
       </c>
       <c r="C32" s="8" t="inlineStr">
@@ -1270,7 +1270,7 @@
       </c>
       <c r="B40" s="7" t="inlineStr">
         <is>
-          <t>📖 Skills File Structure &amp; Organization</t>
+          <t>📖 Skill Anatomy, Progressive Loading &amp; the 6-Step Framework</t>
         </is>
       </c>
       <c r="C40" s="8" t="inlineStr">
@@ -1302,7 +1302,7 @@
       </c>
       <c r="B42" s="7" t="inlineStr">
         <is>
-          <t>🔨 Create the Skills from the Video</t>
+          <t>🔨 Install the Skill Builder &amp; Create Your First Skill</t>
         </is>
       </c>
       <c r="C42" s="8" t="inlineStr">
@@ -1324,7 +1324,7 @@
       </c>
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>🔨 Create Your Own Custom Skill</t>
+          <t>🔨 Create a Custom Skill for Something You Do Repeatedly</t>
         </is>
       </c>
       <c r="C43" s="8" t="inlineStr">
@@ -1356,7 +1356,7 @@
       </c>
       <c r="B45" s="7" t="inlineStr">
         <is>
-          <t>📖 Advanced Skill Patterns</t>
+          <t>📖 Global Skills, Token Optimization &amp; Advanced Front Matter</t>
         </is>
       </c>
       <c r="C45" s="8" t="inlineStr">
@@ -1474,7 +1474,7 @@
       </c>
       <c r="B53" s="7" t="inlineStr">
         <is>
-          <t>📖 From Local to Live: Deployment Concepts</t>
+          <t>📖 From Local to Cloud: The Deployment Pipeline</t>
         </is>
       </c>
       <c r="C53" s="8" t="inlineStr">
@@ -1506,7 +1506,7 @@
       </c>
       <c r="B55" s="7" t="inlineStr">
         <is>
-          <t>🔨 Build and Deploy Nate's Automation</t>
+          <t>🔨 Build and Deploy an Automation to Trigger.dev</t>
         </is>
       </c>
       <c r="C55" s="8" t="inlineStr">
@@ -1528,7 +1528,7 @@
       </c>
       <c r="B56" s="7" t="inlineStr">
         <is>
-          <t>🔨 Deploy Your Own Automation</t>
+          <t>🔨 Deploy a Second Automation or Improve the First</t>
         </is>
       </c>
       <c r="C56" s="8" t="inlineStr">
@@ -1560,7 +1560,7 @@
       </c>
       <c r="B58" s="7" t="inlineStr">
         <is>
-          <t>📖 Environment Variables and Production Config</t>
+          <t>📖 Dev vs Production, Retries &amp; Agentic Tasks</t>
         </is>
       </c>
       <c r="C58" s="8" t="inlineStr">
@@ -1614,7 +1614,7 @@
       </c>
       <c r="B61" s="7" t="inlineStr">
         <is>
-          <t>📣 Share Your Deployed Project</t>
+          <t>📣 Share Your Deployed Automation</t>
         </is>
       </c>
       <c r="C61" s="8" t="inlineStr">
@@ -1656,7 +1656,7 @@
       </c>
       <c r="B65" s="7" t="inlineStr">
         <is>
-          <t>🎬 Watch: Website Build</t>
+          <t>🎬 Watch: Website Build — 5 Hacks</t>
         </is>
       </c>
       <c r="C65" s="8" t="inlineStr">
@@ -1678,7 +1678,7 @@
       </c>
       <c r="B66" s="7" t="inlineStr">
         <is>
-          <t>📖 Web Development Approach with Claude Code</t>
+          <t>📖 The Front-End Skill, Screenshot Loop &amp; Deploy Pipeline</t>
         </is>
       </c>
       <c r="C66" s="8" t="inlineStr">
@@ -1710,7 +1710,7 @@
       </c>
       <c r="B68" s="7" t="inlineStr">
         <is>
-          <t>🔨 Build the Website from the Video</t>
+          <t>🔨 Build a Professional Landing Page</t>
         </is>
       </c>
       <c r="C68" s="8" t="inlineStr">
@@ -1732,7 +1732,7 @@
       </c>
       <c r="B69" s="7" t="inlineStr">
         <is>
-          <t>🔨 Customize and Make It Yours</t>
+          <t>🔨 Clone an Inspiration Site &amp; Customize</t>
         </is>
       </c>
       <c r="C69" s="8" t="inlineStr">
@@ -1764,7 +1764,7 @@
       </c>
       <c r="B71" s="7" t="inlineStr">
         <is>
-          <t>📖 Responsive Design and Deployment</t>
+          <t>📖 Vercel Deployment &amp; When to Disable Screenshots</t>
         </is>
       </c>
       <c r="C71" s="8" t="inlineStr">
@@ -1860,7 +1860,7 @@
       </c>
       <c r="B78" s="7" t="inlineStr">
         <is>
-          <t>🎬 Watch: Scheduled Automations</t>
+          <t>🎬 Watch: Scheduled Tasks in Claude Code</t>
         </is>
       </c>
       <c r="C78" s="8" t="inlineStr">
@@ -1882,7 +1882,7 @@
       </c>
       <c r="B79" s="7" t="inlineStr">
         <is>
-          <t>🎬 Watch: Loop — Recurring Automation Patterns</t>
+          <t>🎬 Watch: Loop — Recurring Tasks Within a Session</t>
         </is>
       </c>
       <c r="C79" s="8" t="inlineStr">
@@ -1904,7 +1904,7 @@
       </c>
       <c r="B80" s="7" t="inlineStr">
         <is>
-          <t>📖 Scheduling Concepts: Cron, Intervals &amp; Triggers</t>
+          <t>📖 Scheduled Tasks vs Loops: When to Use Which</t>
         </is>
       </c>
       <c r="C80" s="8" t="inlineStr">
@@ -1936,7 +1936,7 @@
       </c>
       <c r="B82" s="7" t="inlineStr">
         <is>
-          <t>🔨 Build the Scheduled Automation from the Videos</t>
+          <t>🔨 Create a Scheduled Task and a Loop</t>
         </is>
       </c>
       <c r="C82" s="8" t="inlineStr">
@@ -1958,7 +1958,7 @@
       </c>
       <c r="B83" s="7" t="inlineStr">
         <is>
-          <t>🔨 Build Your Own Recurring Automation</t>
+          <t>🔨 Build a Self-Improving Scheduled Automation</t>
         </is>
       </c>
       <c r="C83" s="8" t="inlineStr">
@@ -1990,7 +1990,7 @@
       </c>
       <c r="B85" s="7" t="inlineStr">
         <is>
-          <t>📖 Error Handling for Recurring Tasks</t>
+          <t>📖 Permissions, Notifications &amp; Safety for Autonomous Tasks</t>
         </is>
       </c>
       <c r="C85" s="8" t="inlineStr">
@@ -2086,7 +2086,7 @@
       </c>
       <c r="B92" s="7" t="inlineStr">
         <is>
-          <t>🎬 Watch: Executive Assistant</t>
+          <t>🎬 Watch: Building an Executive Assistant</t>
         </is>
       </c>
       <c r="C92" s="8" t="inlineStr">
@@ -2108,7 +2108,7 @@
       </c>
       <c r="B93" s="7" t="inlineStr">
         <is>
-          <t>📖 Multi-Component System Architecture</t>
+          <t>📖 The 4-Phase Framework: Home, Life, Hands, Growth</t>
         </is>
       </c>
       <c r="C93" s="8" t="inlineStr">
@@ -2140,7 +2140,7 @@
       </c>
       <c r="B95" s="7" t="inlineStr">
         <is>
-          <t>🔨 Build the Executive Assistant from the Video</t>
+          <t>🔨 Build Your Executive Assistant</t>
         </is>
       </c>
       <c r="C95" s="8" t="inlineStr">
@@ -2162,7 +2162,7 @@
       </c>
       <c r="B96" s="7" t="inlineStr">
         <is>
-          <t>🔨 Add Your Own Feature</t>
+          <t>🔨 Add Your Own Skills and Sub-Agents</t>
         </is>
       </c>
       <c r="C96" s="8" t="inlineStr">
@@ -2194,7 +2194,7 @@
       </c>
       <c r="B98" s="7" t="inlineStr">
         <is>
-          <t>📖 Production Polish</t>
+          <t>📖 Token Management, Sub-Agents &amp; Growing Your EA</t>
         </is>
       </c>
       <c r="C98" s="8" t="inlineStr">

</xml_diff>